<commit_message>
Tarnoc v2: remove 'Why we did not sell more' row and its Dashboard line
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Tarnoc_v2_2026-09-01.xlsx
+++ b/models/Tarnoc_v2_2026-09-01.xlsx
@@ -175,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -347,12 +347,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="170" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1263,13 +1257,6 @@
     <row r="27">
       <c r="C27" s="14" t="inlineStr">
         <is>
-          <t>Revenue Forecast row 35 names which of the three stopped us in each month, and the Dashboard shows it by year.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="C28" s="14" t="inlineStr">
-        <is>
           <t>There is no market size or market share anywhere in the model.</t>
         </is>
       </c>
@@ -18568,7 +18555,7 @@
     <row r="2">
       <c r="B2" s="16" t="inlineStr">
         <is>
-          <t>Units sold is an output: marketing spend generates orders, selling and build capacity cap them, and row 35 says which one bit.</t>
+          <t>Units sold is an output: marketing spend generates orders, and selling and build capacity cap them.</t>
         </is>
       </c>
     </row>
@@ -25126,541 +25113,274 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>Why we did not sell more</t>
-        </is>
-      </c>
-      <c r="E35" s="67">
-        <f>IF(E34&gt;=E31-0.5,"Build capacity",IF(E34&gt;=E22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="F35" s="67">
-        <f>IF(F34&gt;=F31-0.5,"Build capacity",IF(F34&gt;=F22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="G35" s="67">
-        <f>IF(G34&gt;=G31-0.5,"Build capacity",IF(G34&gt;=G22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="H35" s="67">
-        <f>IF(H34&gt;=H31-0.5,"Build capacity",IF(H34&gt;=H22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="I35" s="67">
-        <f>IF(I34&gt;=I31-0.5,"Build capacity",IF(I34&gt;=I22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="J35" s="67">
-        <f>IF(J34&gt;=J31-0.5,"Build capacity",IF(J34&gt;=J22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="K35" s="67">
-        <f>IF(K34&gt;=K31-0.5,"Build capacity",IF(K34&gt;=K22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="L35" s="67">
-        <f>IF(L34&gt;=L31-0.5,"Build capacity",IF(L34&gt;=L22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="M35" s="67">
-        <f>IF(M34&gt;=M31-0.5,"Build capacity",IF(M34&gt;=M22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="N35" s="67">
-        <f>IF(N34&gt;=N31-0.5,"Build capacity",IF(N34&gt;=N22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="O35" s="67">
-        <f>IF(O34&gt;=O31-0.5,"Build capacity",IF(O34&gt;=O22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="P35" s="67">
-        <f>IF(P34&gt;=P31-0.5,"Build capacity",IF(P34&gt;=P22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="Q35" s="67">
-        <f>IF(Q34&gt;=Q31-0.5,"Build capacity",IF(Q34&gt;=Q22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="R35" s="67">
-        <f>IF(R34&gt;=R31-0.5,"Build capacity",IF(R34&gt;=R22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="S35" s="67">
-        <f>IF(S34&gt;=S31-0.5,"Build capacity",IF(S34&gt;=S22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="T35" s="67">
-        <f>IF(T34&gt;=T31-0.5,"Build capacity",IF(T34&gt;=T22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="U35" s="67">
-        <f>IF(U34&gt;=U31-0.5,"Build capacity",IF(U34&gt;=U22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="V35" s="67">
-        <f>IF(V34&gt;=V31-0.5,"Build capacity",IF(V34&gt;=V22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="W35" s="67">
-        <f>IF(W34&gt;=W31-0.5,"Build capacity",IF(W34&gt;=W22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="X35" s="67">
-        <f>IF(X34&gt;=X31-0.5,"Build capacity",IF(X34&gt;=X22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="Y35" s="67">
-        <f>IF(Y34&gt;=Y31-0.5,"Build capacity",IF(Y34&gt;=Y22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="Z35" s="67">
-        <f>IF(Z34&gt;=Z31-0.5,"Build capacity",IF(Z34&gt;=Z22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AA35" s="67">
-        <f>IF(AA34&gt;=AA31-0.5,"Build capacity",IF(AA34&gt;=AA22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AB35" s="67">
-        <f>IF(AB34&gt;=AB31-0.5,"Build capacity",IF(AB34&gt;=AB22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AC35" s="67">
-        <f>IF(AC34&gt;=AC31-0.5,"Build capacity",IF(AC34&gt;=AC22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AD35" s="67">
-        <f>IF(AD34&gt;=AD31-0.5,"Build capacity",IF(AD34&gt;=AD22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AE35" s="67">
-        <f>IF(AE34&gt;=AE31-0.5,"Build capacity",IF(AE34&gt;=AE22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AF35" s="67">
-        <f>IF(AF34&gt;=AF31-0.5,"Build capacity",IF(AF34&gt;=AF22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AG35" s="67">
-        <f>IF(AG34&gt;=AG31-0.5,"Build capacity",IF(AG34&gt;=AG22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AH35" s="67">
-        <f>IF(AH34&gt;=AH31-0.5,"Build capacity",IF(AH34&gt;=AH22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AI35" s="67">
-        <f>IF(AI34&gt;=AI31-0.5,"Build capacity",IF(AI34&gt;=AI22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AJ35" s="67">
-        <f>IF(AJ34&gt;=AJ31-0.5,"Build capacity",IF(AJ34&gt;=AJ22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AK35" s="67">
-        <f>IF(AK34&gt;=AK31-0.5,"Build capacity",IF(AK34&gt;=AK22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AL35" s="67">
-        <f>IF(AL34&gt;=AL31-0.5,"Build capacity",IF(AL34&gt;=AL22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AM35" s="67">
-        <f>IF(AM34&gt;=AM31-0.5,"Build capacity",IF(AM34&gt;=AM22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AN35" s="67">
-        <f>IF(AN34&gt;=AN31-0.5,"Build capacity",IF(AN34&gt;=AN22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AO35" s="67">
-        <f>IF(AO34&gt;=AO31-0.5,"Build capacity",IF(AO34&gt;=AO22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AP35" s="67">
-        <f>IF(AP34&gt;=AP31-0.5,"Build capacity",IF(AP34&gt;=AP22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AQ35" s="67">
-        <f>IF(AQ34&gt;=AQ31-0.5,"Build capacity",IF(AQ34&gt;=AQ22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AR35" s="67">
-        <f>IF(AR34&gt;=AR31-0.5,"Build capacity",IF(AR34&gt;=AR22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AS35" s="67">
-        <f>IF(AS34&gt;=AS31-0.5,"Build capacity",IF(AS34&gt;=AS22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AT35" s="67">
-        <f>IF(AT34&gt;=AT31-0.5,"Build capacity",IF(AT34&gt;=AT22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AU35" s="67">
-        <f>IF(AU34&gt;=AU31-0.5,"Build capacity",IF(AU34&gt;=AU22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AV35" s="67">
-        <f>IF(AV34&gt;=AV31-0.5,"Build capacity",IF(AV34&gt;=AV22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AW35" s="67">
-        <f>IF(AW34&gt;=AW31-0.5,"Build capacity",IF(AW34&gt;=AW22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AX35" s="67">
-        <f>IF(AX34&gt;=AX31-0.5,"Build capacity",IF(AX34&gt;=AX22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AY35" s="67">
-        <f>IF(AY34&gt;=AY31-0.5,"Build capacity",IF(AY34&gt;=AY22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="AZ35" s="67">
-        <f>IF(AZ34&gt;=AZ31-0.5,"Build capacity",IF(AZ34&gt;=AZ22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="BA35" s="67">
-        <f>IF(BA34&gt;=BA31-0.5,"Build capacity",IF(BA34&gt;=BA22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="BB35" s="67">
-        <f>IF(BB34&gt;=BB31-0.5,"Build capacity",IF(BB34&gt;=BB22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="BC35" s="67">
-        <f>IF(BC34&gt;=BC31-0.5,"Build capacity",IF(BC34&gt;=BC22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="BD35" s="67">
-        <f>IF(BD34&gt;=BD31-0.5,"Build capacity",IF(BD34&gt;=BD22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="BE35" s="67">
-        <f>IF(BE34&gt;=BE31-0.5,"Build capacity",IF(BE34&gt;=BE22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="BF35" s="67">
-        <f>IF(BF34&gt;=BF31-0.5,"Build capacity",IF(BF34&gt;=BF22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="BG35" s="67">
-        <f>IF(BG34&gt;=BG31-0.5,"Build capacity",IF(BG34&gt;=BG22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="BH35" s="67">
-        <f>IF(BH34&gt;=BH31-0.5,"Build capacity",IF(BH34&gt;=BH22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="BI35" s="67">
-        <f>IF(BI34&gt;=BI31-0.5,"Build capacity",IF(BI34&gt;=BI22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="BJ35" s="67">
-        <f>IF(BJ34&gt;=BJ31-0.5,"Build capacity",IF(BJ34&gt;=BJ22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="BK35" s="67">
-        <f>IF(BK34&gt;=BK31-0.5,"Build capacity",IF(BK34&gt;=BK22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="BL35" s="67">
-        <f>IF(BL34&gt;=BL31-0.5,"Build capacity",IF(BL34&gt;=BL22-0.5,"Selling capacity","Demand"))</f>
-        <v/>
-      </c>
-      <c r="BN35" s="68">
-        <f>P35</f>
-        <v/>
-      </c>
-      <c r="BO35" s="68">
-        <f>AB35</f>
-        <v/>
-      </c>
-      <c r="BP35" s="68">
-        <f>AN35</f>
-        <v/>
-      </c>
-      <c r="BQ35" s="68">
-        <f>AZ35</f>
-        <v/>
-      </c>
-      <c r="BR35" s="68">
-        <f>BL35</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="47" t="inlineStr">
+      <c r="B35" s="47" t="inlineStr">
         <is>
           <t>Build capacity used</t>
         </is>
       </c>
-      <c r="C36" s="42" t="inlineStr">
+      <c r="C35" s="42" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E36" s="64">
+      <c r="E35" s="64">
         <f>IFERROR(E34/E31,0)</f>
         <v/>
       </c>
-      <c r="F36" s="64">
+      <c r="F35" s="64">
         <f>IFERROR(F34/F31,0)</f>
         <v/>
       </c>
-      <c r="G36" s="64">
+      <c r="G35" s="64">
         <f>IFERROR(G34/G31,0)</f>
         <v/>
       </c>
-      <c r="H36" s="64">
+      <c r="H35" s="64">
         <f>IFERROR(H34/H31,0)</f>
         <v/>
       </c>
-      <c r="I36" s="64">
+      <c r="I35" s="64">
         <f>IFERROR(I34/I31,0)</f>
         <v/>
       </c>
-      <c r="J36" s="64">
+      <c r="J35" s="64">
         <f>IFERROR(J34/J31,0)</f>
         <v/>
       </c>
-      <c r="K36" s="64">
+      <c r="K35" s="64">
         <f>IFERROR(K34/K31,0)</f>
         <v/>
       </c>
-      <c r="L36" s="64">
+      <c r="L35" s="64">
         <f>IFERROR(L34/L31,0)</f>
         <v/>
       </c>
-      <c r="M36" s="64">
+      <c r="M35" s="64">
         <f>IFERROR(M34/M31,0)</f>
         <v/>
       </c>
-      <c r="N36" s="64">
+      <c r="N35" s="64">
         <f>IFERROR(N34/N31,0)</f>
         <v/>
       </c>
-      <c r="O36" s="64">
+      <c r="O35" s="64">
         <f>IFERROR(O34/O31,0)</f>
         <v/>
       </c>
-      <c r="P36" s="64">
+      <c r="P35" s="64">
         <f>IFERROR(P34/P31,0)</f>
         <v/>
       </c>
-      <c r="Q36" s="64">
+      <c r="Q35" s="64">
         <f>IFERROR(Q34/Q31,0)</f>
         <v/>
       </c>
-      <c r="R36" s="64">
+      <c r="R35" s="64">
         <f>IFERROR(R34/R31,0)</f>
         <v/>
       </c>
-      <c r="S36" s="64">
+      <c r="S35" s="64">
         <f>IFERROR(S34/S31,0)</f>
         <v/>
       </c>
-      <c r="T36" s="64">
+      <c r="T35" s="64">
         <f>IFERROR(T34/T31,0)</f>
         <v/>
       </c>
-      <c r="U36" s="64">
+      <c r="U35" s="64">
         <f>IFERROR(U34/U31,0)</f>
         <v/>
       </c>
-      <c r="V36" s="64">
+      <c r="V35" s="64">
         <f>IFERROR(V34/V31,0)</f>
         <v/>
       </c>
-      <c r="W36" s="64">
+      <c r="W35" s="64">
         <f>IFERROR(W34/W31,0)</f>
         <v/>
       </c>
-      <c r="X36" s="64">
+      <c r="X35" s="64">
         <f>IFERROR(X34/X31,0)</f>
         <v/>
       </c>
-      <c r="Y36" s="64">
+      <c r="Y35" s="64">
         <f>IFERROR(Y34/Y31,0)</f>
         <v/>
       </c>
-      <c r="Z36" s="64">
+      <c r="Z35" s="64">
         <f>IFERROR(Z34/Z31,0)</f>
         <v/>
       </c>
-      <c r="AA36" s="64">
+      <c r="AA35" s="64">
         <f>IFERROR(AA34/AA31,0)</f>
         <v/>
       </c>
-      <c r="AB36" s="64">
+      <c r="AB35" s="64">
         <f>IFERROR(AB34/AB31,0)</f>
         <v/>
       </c>
-      <c r="AC36" s="64">
+      <c r="AC35" s="64">
         <f>IFERROR(AC34/AC31,0)</f>
         <v/>
       </c>
-      <c r="AD36" s="64">
+      <c r="AD35" s="64">
         <f>IFERROR(AD34/AD31,0)</f>
         <v/>
       </c>
-      <c r="AE36" s="64">
+      <c r="AE35" s="64">
         <f>IFERROR(AE34/AE31,0)</f>
         <v/>
       </c>
-      <c r="AF36" s="64">
+      <c r="AF35" s="64">
         <f>IFERROR(AF34/AF31,0)</f>
         <v/>
       </c>
-      <c r="AG36" s="64">
+      <c r="AG35" s="64">
         <f>IFERROR(AG34/AG31,0)</f>
         <v/>
       </c>
-      <c r="AH36" s="64">
+      <c r="AH35" s="64">
         <f>IFERROR(AH34/AH31,0)</f>
         <v/>
       </c>
-      <c r="AI36" s="64">
+      <c r="AI35" s="64">
         <f>IFERROR(AI34/AI31,0)</f>
         <v/>
       </c>
-      <c r="AJ36" s="64">
+      <c r="AJ35" s="64">
         <f>IFERROR(AJ34/AJ31,0)</f>
         <v/>
       </c>
-      <c r="AK36" s="64">
+      <c r="AK35" s="64">
         <f>IFERROR(AK34/AK31,0)</f>
         <v/>
       </c>
-      <c r="AL36" s="64">
+      <c r="AL35" s="64">
         <f>IFERROR(AL34/AL31,0)</f>
         <v/>
       </c>
-      <c r="AM36" s="64">
+      <c r="AM35" s="64">
         <f>IFERROR(AM34/AM31,0)</f>
         <v/>
       </c>
-      <c r="AN36" s="64">
+      <c r="AN35" s="64">
         <f>IFERROR(AN34/AN31,0)</f>
         <v/>
       </c>
-      <c r="AO36" s="64">
+      <c r="AO35" s="64">
         <f>IFERROR(AO34/AO31,0)</f>
         <v/>
       </c>
-      <c r="AP36" s="64">
+      <c r="AP35" s="64">
         <f>IFERROR(AP34/AP31,0)</f>
         <v/>
       </c>
-      <c r="AQ36" s="64">
+      <c r="AQ35" s="64">
         <f>IFERROR(AQ34/AQ31,0)</f>
         <v/>
       </c>
-      <c r="AR36" s="64">
+      <c r="AR35" s="64">
         <f>IFERROR(AR34/AR31,0)</f>
         <v/>
       </c>
-      <c r="AS36" s="64">
+      <c r="AS35" s="64">
         <f>IFERROR(AS34/AS31,0)</f>
         <v/>
       </c>
-      <c r="AT36" s="64">
+      <c r="AT35" s="64">
         <f>IFERROR(AT34/AT31,0)</f>
         <v/>
       </c>
-      <c r="AU36" s="64">
+      <c r="AU35" s="64">
         <f>IFERROR(AU34/AU31,0)</f>
         <v/>
       </c>
-      <c r="AV36" s="64">
+      <c r="AV35" s="64">
         <f>IFERROR(AV34/AV31,0)</f>
         <v/>
       </c>
-      <c r="AW36" s="64">
+      <c r="AW35" s="64">
         <f>IFERROR(AW34/AW31,0)</f>
         <v/>
       </c>
-      <c r="AX36" s="64">
+      <c r="AX35" s="64">
         <f>IFERROR(AX34/AX31,0)</f>
         <v/>
       </c>
-      <c r="AY36" s="64">
+      <c r="AY35" s="64">
         <f>IFERROR(AY34/AY31,0)</f>
         <v/>
       </c>
-      <c r="AZ36" s="64">
+      <c r="AZ35" s="64">
         <f>IFERROR(AZ34/AZ31,0)</f>
         <v/>
       </c>
-      <c r="BA36" s="64">
+      <c r="BA35" s="64">
         <f>IFERROR(BA34/BA31,0)</f>
         <v/>
       </c>
-      <c r="BB36" s="64">
+      <c r="BB35" s="64">
         <f>IFERROR(BB34/BB31,0)</f>
         <v/>
       </c>
-      <c r="BC36" s="64">
+      <c r="BC35" s="64">
         <f>IFERROR(BC34/BC31,0)</f>
         <v/>
       </c>
-      <c r="BD36" s="64">
+      <c r="BD35" s="64">
         <f>IFERROR(BD34/BD31,0)</f>
         <v/>
       </c>
-      <c r="BE36" s="64">
+      <c r="BE35" s="64">
         <f>IFERROR(BE34/BE31,0)</f>
         <v/>
       </c>
-      <c r="BF36" s="64">
+      <c r="BF35" s="64">
         <f>IFERROR(BF34/BF31,0)</f>
         <v/>
       </c>
-      <c r="BG36" s="64">
+      <c r="BG35" s="64">
         <f>IFERROR(BG34/BG31,0)</f>
         <v/>
       </c>
-      <c r="BH36" s="64">
+      <c r="BH35" s="64">
         <f>IFERROR(BH34/BH31,0)</f>
         <v/>
       </c>
-      <c r="BI36" s="64">
+      <c r="BI35" s="64">
         <f>IFERROR(BI34/BI31,0)</f>
         <v/>
       </c>
-      <c r="BJ36" s="64">
+      <c r="BJ35" s="64">
         <f>IFERROR(BJ34/BJ31,0)</f>
         <v/>
       </c>
-      <c r="BK36" s="64">
+      <c r="BK35" s="64">
         <f>IFERROR(BK34/BK31,0)</f>
         <v/>
       </c>
-      <c r="BL36" s="64">
+      <c r="BL35" s="64">
         <f>IFERROR(BL34/BL31,0)</f>
         <v/>
       </c>
-      <c r="BN36" s="65">
-        <f>IFERROR(AVERAGE(E36:P36),0)</f>
-        <v/>
-      </c>
-      <c r="BO36" s="65">
-        <f>IFERROR(AVERAGE(Q36:AB36),0)</f>
-        <v/>
-      </c>
-      <c r="BP36" s="65">
-        <f>IFERROR(AVERAGE(AC36:AN36),0)</f>
-        <v/>
-      </c>
-      <c r="BQ36" s="65">
-        <f>IFERROR(AVERAGE(AO36:AZ36),0)</f>
-        <v/>
-      </c>
-      <c r="BR36" s="65">
-        <f>IFERROR(AVERAGE(BA36:BL36),0)</f>
+      <c r="BN35" s="65">
+        <f>IFERROR(AVERAGE(E35:P35),0)</f>
+        <v/>
+      </c>
+      <c r="BO35" s="65">
+        <f>IFERROR(AVERAGE(Q35:AB35),0)</f>
+        <v/>
+      </c>
+      <c r="BP35" s="65">
+        <f>IFERROR(AVERAGE(AC35:AN35),0)</f>
+        <v/>
+      </c>
+      <c r="BQ35" s="65">
+        <f>IFERROR(AVERAGE(AO35:AZ35),0)</f>
+        <v/>
+      </c>
+      <c r="BR35" s="65">
+        <f>IFERROR(AVERAGE(BA35:BL35),0)</f>
         <v/>
       </c>
     </row>
@@ -41510,263 +41230,263 @@
           <t>FTE</t>
         </is>
       </c>
-      <c r="E7" s="69">
+      <c r="E7" s="67">
         <f>'Revenue Forecast'!E23</f>
         <v/>
       </c>
-      <c r="F7" s="69">
+      <c r="F7" s="67">
         <f>'Revenue Forecast'!F23</f>
         <v/>
       </c>
-      <c r="G7" s="69">
+      <c r="G7" s="67">
         <f>'Revenue Forecast'!G23</f>
         <v/>
       </c>
-      <c r="H7" s="69">
+      <c r="H7" s="67">
         <f>'Revenue Forecast'!H23</f>
         <v/>
       </c>
-      <c r="I7" s="69">
+      <c r="I7" s="67">
         <f>'Revenue Forecast'!I23</f>
         <v/>
       </c>
-      <c r="J7" s="69">
+      <c r="J7" s="67">
         <f>'Revenue Forecast'!J23</f>
         <v/>
       </c>
-      <c r="K7" s="69">
+      <c r="K7" s="67">
         <f>'Revenue Forecast'!K23</f>
         <v/>
       </c>
-      <c r="L7" s="69">
+      <c r="L7" s="67">
         <f>'Revenue Forecast'!L23</f>
         <v/>
       </c>
-      <c r="M7" s="69">
+      <c r="M7" s="67">
         <f>'Revenue Forecast'!M23</f>
         <v/>
       </c>
-      <c r="N7" s="69">
+      <c r="N7" s="67">
         <f>'Revenue Forecast'!N23</f>
         <v/>
       </c>
-      <c r="O7" s="69">
+      <c r="O7" s="67">
         <f>'Revenue Forecast'!O23</f>
         <v/>
       </c>
-      <c r="P7" s="69">
+      <c r="P7" s="67">
         <f>'Revenue Forecast'!P23</f>
         <v/>
       </c>
-      <c r="Q7" s="69">
+      <c r="Q7" s="67">
         <f>'Revenue Forecast'!Q23</f>
         <v/>
       </c>
-      <c r="R7" s="69">
+      <c r="R7" s="67">
         <f>'Revenue Forecast'!R23</f>
         <v/>
       </c>
-      <c r="S7" s="69">
+      <c r="S7" s="67">
         <f>'Revenue Forecast'!S23</f>
         <v/>
       </c>
-      <c r="T7" s="69">
+      <c r="T7" s="67">
         <f>'Revenue Forecast'!T23</f>
         <v/>
       </c>
-      <c r="U7" s="69">
+      <c r="U7" s="67">
         <f>'Revenue Forecast'!U23</f>
         <v/>
       </c>
-      <c r="V7" s="69">
+      <c r="V7" s="67">
         <f>'Revenue Forecast'!V23</f>
         <v/>
       </c>
-      <c r="W7" s="69">
+      <c r="W7" s="67">
         <f>'Revenue Forecast'!W23</f>
         <v/>
       </c>
-      <c r="X7" s="69">
+      <c r="X7" s="67">
         <f>'Revenue Forecast'!X23</f>
         <v/>
       </c>
-      <c r="Y7" s="69">
+      <c r="Y7" s="67">
         <f>'Revenue Forecast'!Y23</f>
         <v/>
       </c>
-      <c r="Z7" s="69">
+      <c r="Z7" s="67">
         <f>'Revenue Forecast'!Z23</f>
         <v/>
       </c>
-      <c r="AA7" s="69">
+      <c r="AA7" s="67">
         <f>'Revenue Forecast'!AA23</f>
         <v/>
       </c>
-      <c r="AB7" s="69">
+      <c r="AB7" s="67">
         <f>'Revenue Forecast'!AB23</f>
         <v/>
       </c>
-      <c r="AC7" s="69">
+      <c r="AC7" s="67">
         <f>'Revenue Forecast'!AC23</f>
         <v/>
       </c>
-      <c r="AD7" s="69">
+      <c r="AD7" s="67">
         <f>'Revenue Forecast'!AD23</f>
         <v/>
       </c>
-      <c r="AE7" s="69">
+      <c r="AE7" s="67">
         <f>'Revenue Forecast'!AE23</f>
         <v/>
       </c>
-      <c r="AF7" s="69">
+      <c r="AF7" s="67">
         <f>'Revenue Forecast'!AF23</f>
         <v/>
       </c>
-      <c r="AG7" s="69">
+      <c r="AG7" s="67">
         <f>'Revenue Forecast'!AG23</f>
         <v/>
       </c>
-      <c r="AH7" s="69">
+      <c r="AH7" s="67">
         <f>'Revenue Forecast'!AH23</f>
         <v/>
       </c>
-      <c r="AI7" s="69">
+      <c r="AI7" s="67">
         <f>'Revenue Forecast'!AI23</f>
         <v/>
       </c>
-      <c r="AJ7" s="69">
+      <c r="AJ7" s="67">
         <f>'Revenue Forecast'!AJ23</f>
         <v/>
       </c>
-      <c r="AK7" s="69">
+      <c r="AK7" s="67">
         <f>'Revenue Forecast'!AK23</f>
         <v/>
       </c>
-      <c r="AL7" s="69">
+      <c r="AL7" s="67">
         <f>'Revenue Forecast'!AL23</f>
         <v/>
       </c>
-      <c r="AM7" s="69">
+      <c r="AM7" s="67">
         <f>'Revenue Forecast'!AM23</f>
         <v/>
       </c>
-      <c r="AN7" s="69">
+      <c r="AN7" s="67">
         <f>'Revenue Forecast'!AN23</f>
         <v/>
       </c>
-      <c r="AO7" s="69">
+      <c r="AO7" s="67">
         <f>'Revenue Forecast'!AO23</f>
         <v/>
       </c>
-      <c r="AP7" s="69">
+      <c r="AP7" s="67">
         <f>'Revenue Forecast'!AP23</f>
         <v/>
       </c>
-      <c r="AQ7" s="69">
+      <c r="AQ7" s="67">
         <f>'Revenue Forecast'!AQ23</f>
         <v/>
       </c>
-      <c r="AR7" s="69">
+      <c r="AR7" s="67">
         <f>'Revenue Forecast'!AR23</f>
         <v/>
       </c>
-      <c r="AS7" s="69">
+      <c r="AS7" s="67">
         <f>'Revenue Forecast'!AS23</f>
         <v/>
       </c>
-      <c r="AT7" s="69">
+      <c r="AT7" s="67">
         <f>'Revenue Forecast'!AT23</f>
         <v/>
       </c>
-      <c r="AU7" s="69">
+      <c r="AU7" s="67">
         <f>'Revenue Forecast'!AU23</f>
         <v/>
       </c>
-      <c r="AV7" s="69">
+      <c r="AV7" s="67">
         <f>'Revenue Forecast'!AV23</f>
         <v/>
       </c>
-      <c r="AW7" s="69">
+      <c r="AW7" s="67">
         <f>'Revenue Forecast'!AW23</f>
         <v/>
       </c>
-      <c r="AX7" s="69">
+      <c r="AX7" s="67">
         <f>'Revenue Forecast'!AX23</f>
         <v/>
       </c>
-      <c r="AY7" s="69">
+      <c r="AY7" s="67">
         <f>'Revenue Forecast'!AY23</f>
         <v/>
       </c>
-      <c r="AZ7" s="69">
+      <c r="AZ7" s="67">
         <f>'Revenue Forecast'!AZ23</f>
         <v/>
       </c>
-      <c r="BA7" s="69">
+      <c r="BA7" s="67">
         <f>'Revenue Forecast'!BA23</f>
         <v/>
       </c>
-      <c r="BB7" s="69">
+      <c r="BB7" s="67">
         <f>'Revenue Forecast'!BB23</f>
         <v/>
       </c>
-      <c r="BC7" s="69">
+      <c r="BC7" s="67">
         <f>'Revenue Forecast'!BC23</f>
         <v/>
       </c>
-      <c r="BD7" s="69">
+      <c r="BD7" s="67">
         <f>'Revenue Forecast'!BD23</f>
         <v/>
       </c>
-      <c r="BE7" s="69">
+      <c r="BE7" s="67">
         <f>'Revenue Forecast'!BE23</f>
         <v/>
       </c>
-      <c r="BF7" s="69">
+      <c r="BF7" s="67">
         <f>'Revenue Forecast'!BF23</f>
         <v/>
       </c>
-      <c r="BG7" s="69">
+      <c r="BG7" s="67">
         <f>'Revenue Forecast'!BG23</f>
         <v/>
       </c>
-      <c r="BH7" s="69">
+      <c r="BH7" s="67">
         <f>'Revenue Forecast'!BH23</f>
         <v/>
       </c>
-      <c r="BI7" s="69">
+      <c r="BI7" s="67">
         <f>'Revenue Forecast'!BI23</f>
         <v/>
       </c>
-      <c r="BJ7" s="69">
+      <c r="BJ7" s="67">
         <f>'Revenue Forecast'!BJ23</f>
         <v/>
       </c>
-      <c r="BK7" s="69">
+      <c r="BK7" s="67">
         <f>'Revenue Forecast'!BK23</f>
         <v/>
       </c>
-      <c r="BL7" s="69">
+      <c r="BL7" s="67">
         <f>'Revenue Forecast'!BL23</f>
         <v/>
       </c>
-      <c r="BN7" s="70">
+      <c r="BN7" s="68">
         <f>P7</f>
         <v/>
       </c>
-      <c r="BO7" s="70">
+      <c r="BO7" s="68">
         <f>AB7</f>
         <v/>
       </c>
-      <c r="BP7" s="70">
+      <c r="BP7" s="68">
         <f>AN7</f>
         <v/>
       </c>
-      <c r="BQ7" s="70">
+      <c r="BQ7" s="68">
         <f>AZ7</f>
         <v/>
       </c>
-      <c r="BR7" s="70">
+      <c r="BR7" s="68">
         <f>BL7</f>
         <v/>
       </c>
@@ -45893,264 +45613,264 @@
         </is>
       </c>
       <c r="D23" s="1" t="n"/>
-      <c r="E23" s="71">
+      <c r="E23" s="69">
         <f>E21+E22</f>
         <v/>
       </c>
-      <c r="F23" s="71">
+      <c r="F23" s="69">
         <f>F21+F22</f>
         <v/>
       </c>
-      <c r="G23" s="71">
+      <c r="G23" s="69">
         <f>G21+G22</f>
         <v/>
       </c>
-      <c r="H23" s="71">
+      <c r="H23" s="69">
         <f>H21+H22</f>
         <v/>
       </c>
-      <c r="I23" s="71">
+      <c r="I23" s="69">
         <f>I21+I22</f>
         <v/>
       </c>
-      <c r="J23" s="71">
+      <c r="J23" s="69">
         <f>J21+J22</f>
         <v/>
       </c>
-      <c r="K23" s="71">
+      <c r="K23" s="69">
         <f>K21+K22</f>
         <v/>
       </c>
-      <c r="L23" s="71">
+      <c r="L23" s="69">
         <f>L21+L22</f>
         <v/>
       </c>
-      <c r="M23" s="71">
+      <c r="M23" s="69">
         <f>M21+M22</f>
         <v/>
       </c>
-      <c r="N23" s="71">
+      <c r="N23" s="69">
         <f>N21+N22</f>
         <v/>
       </c>
-      <c r="O23" s="71">
+      <c r="O23" s="69">
         <f>O21+O22</f>
         <v/>
       </c>
-      <c r="P23" s="71">
+      <c r="P23" s="69">
         <f>P21+P22</f>
         <v/>
       </c>
-      <c r="Q23" s="71">
+      <c r="Q23" s="69">
         <f>Q21+Q22</f>
         <v/>
       </c>
-      <c r="R23" s="71">
+      <c r="R23" s="69">
         <f>R21+R22</f>
         <v/>
       </c>
-      <c r="S23" s="71">
+      <c r="S23" s="69">
         <f>S21+S22</f>
         <v/>
       </c>
-      <c r="T23" s="71">
+      <c r="T23" s="69">
         <f>T21+T22</f>
         <v/>
       </c>
-      <c r="U23" s="71">
+      <c r="U23" s="69">
         <f>U21+U22</f>
         <v/>
       </c>
-      <c r="V23" s="71">
+      <c r="V23" s="69">
         <f>V21+V22</f>
         <v/>
       </c>
-      <c r="W23" s="71">
+      <c r="W23" s="69">
         <f>W21+W22</f>
         <v/>
       </c>
-      <c r="X23" s="71">
+      <c r="X23" s="69">
         <f>X21+X22</f>
         <v/>
       </c>
-      <c r="Y23" s="71">
+      <c r="Y23" s="69">
         <f>Y21+Y22</f>
         <v/>
       </c>
-      <c r="Z23" s="71">
+      <c r="Z23" s="69">
         <f>Z21+Z22</f>
         <v/>
       </c>
-      <c r="AA23" s="71">
+      <c r="AA23" s="69">
         <f>AA21+AA22</f>
         <v/>
       </c>
-      <c r="AB23" s="71">
+      <c r="AB23" s="69">
         <f>AB21+AB22</f>
         <v/>
       </c>
-      <c r="AC23" s="71">
+      <c r="AC23" s="69">
         <f>AC21+AC22</f>
         <v/>
       </c>
-      <c r="AD23" s="71">
+      <c r="AD23" s="69">
         <f>AD21+AD22</f>
         <v/>
       </c>
-      <c r="AE23" s="71">
+      <c r="AE23" s="69">
         <f>AE21+AE22</f>
         <v/>
       </c>
-      <c r="AF23" s="71">
+      <c r="AF23" s="69">
         <f>AF21+AF22</f>
         <v/>
       </c>
-      <c r="AG23" s="71">
+      <c r="AG23" s="69">
         <f>AG21+AG22</f>
         <v/>
       </c>
-      <c r="AH23" s="71">
+      <c r="AH23" s="69">
         <f>AH21+AH22</f>
         <v/>
       </c>
-      <c r="AI23" s="71">
+      <c r="AI23" s="69">
         <f>AI21+AI22</f>
         <v/>
       </c>
-      <c r="AJ23" s="71">
+      <c r="AJ23" s="69">
         <f>AJ21+AJ22</f>
         <v/>
       </c>
-      <c r="AK23" s="71">
+      <c r="AK23" s="69">
         <f>AK21+AK22</f>
         <v/>
       </c>
-      <c r="AL23" s="71">
+      <c r="AL23" s="69">
         <f>AL21+AL22</f>
         <v/>
       </c>
-      <c r="AM23" s="71">
+      <c r="AM23" s="69">
         <f>AM21+AM22</f>
         <v/>
       </c>
-      <c r="AN23" s="71">
+      <c r="AN23" s="69">
         <f>AN21+AN22</f>
         <v/>
       </c>
-      <c r="AO23" s="71">
+      <c r="AO23" s="69">
         <f>AO21+AO22</f>
         <v/>
       </c>
-      <c r="AP23" s="71">
+      <c r="AP23" s="69">
         <f>AP21+AP22</f>
         <v/>
       </c>
-      <c r="AQ23" s="71">
+      <c r="AQ23" s="69">
         <f>AQ21+AQ22</f>
         <v/>
       </c>
-      <c r="AR23" s="71">
+      <c r="AR23" s="69">
         <f>AR21+AR22</f>
         <v/>
       </c>
-      <c r="AS23" s="71">
+      <c r="AS23" s="69">
         <f>AS21+AS22</f>
         <v/>
       </c>
-      <c r="AT23" s="71">
+      <c r="AT23" s="69">
         <f>AT21+AT22</f>
         <v/>
       </c>
-      <c r="AU23" s="71">
+      <c r="AU23" s="69">
         <f>AU21+AU22</f>
         <v/>
       </c>
-      <c r="AV23" s="71">
+      <c r="AV23" s="69">
         <f>AV21+AV22</f>
         <v/>
       </c>
-      <c r="AW23" s="71">
+      <c r="AW23" s="69">
         <f>AW21+AW22</f>
         <v/>
       </c>
-      <c r="AX23" s="71">
+      <c r="AX23" s="69">
         <f>AX21+AX22</f>
         <v/>
       </c>
-      <c r="AY23" s="71">
+      <c r="AY23" s="69">
         <f>AY21+AY22</f>
         <v/>
       </c>
-      <c r="AZ23" s="71">
+      <c r="AZ23" s="69">
         <f>AZ21+AZ22</f>
         <v/>
       </c>
-      <c r="BA23" s="71">
+      <c r="BA23" s="69">
         <f>BA21+BA22</f>
         <v/>
       </c>
-      <c r="BB23" s="71">
+      <c r="BB23" s="69">
         <f>BB21+BB22</f>
         <v/>
       </c>
-      <c r="BC23" s="71">
+      <c r="BC23" s="69">
         <f>BC21+BC22</f>
         <v/>
       </c>
-      <c r="BD23" s="71">
+      <c r="BD23" s="69">
         <f>BD21+BD22</f>
         <v/>
       </c>
-      <c r="BE23" s="71">
+      <c r="BE23" s="69">
         <f>BE21+BE22</f>
         <v/>
       </c>
-      <c r="BF23" s="71">
+      <c r="BF23" s="69">
         <f>BF21+BF22</f>
         <v/>
       </c>
-      <c r="BG23" s="71">
+      <c r="BG23" s="69">
         <f>BG21+BG22</f>
         <v/>
       </c>
-      <c r="BH23" s="71">
+      <c r="BH23" s="69">
         <f>BH21+BH22</f>
         <v/>
       </c>
-      <c r="BI23" s="71">
+      <c r="BI23" s="69">
         <f>BI21+BI22</f>
         <v/>
       </c>
-      <c r="BJ23" s="71">
+      <c r="BJ23" s="69">
         <f>BJ21+BJ22</f>
         <v/>
       </c>
-      <c r="BK23" s="71">
+      <c r="BK23" s="69">
         <f>BK21+BK22</f>
         <v/>
       </c>
-      <c r="BL23" s="71">
+      <c r="BL23" s="69">
         <f>BL21+BL22</f>
         <v/>
       </c>
       <c r="BM23" s="1" t="n"/>
-      <c r="BN23" s="71">
+      <c r="BN23" s="69">
         <f>P23</f>
         <v/>
       </c>
-      <c r="BO23" s="71">
+      <c r="BO23" s="69">
         <f>AB23</f>
         <v/>
       </c>
-      <c r="BP23" s="71">
+      <c r="BP23" s="69">
         <f>AN23</f>
         <v/>
       </c>
-      <c r="BQ23" s="71">
+      <c r="BQ23" s="69">
         <f>AZ23</f>
         <v/>
       </c>
-      <c r="BR23" s="71">
+      <c r="BR23" s="69">
         <f>BL23</f>
         <v/>
       </c>
@@ -47733,112 +47453,80 @@
     <row r="8">
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Why we did not sell more, December</t>
-        </is>
-      </c>
-      <c r="D8" s="67">
-        <f>'Revenue Forecast'!P35</f>
-        <v/>
-      </c>
-      <c r="E8" s="67">
-        <f>'Revenue Forecast'!AB35</f>
-        <v/>
-      </c>
-      <c r="F8" s="67">
-        <f>'Revenue Forecast'!AN35</f>
-        <v/>
-      </c>
-      <c r="G8" s="67">
-        <f>'Revenue Forecast'!AZ35</f>
-        <v/>
-      </c>
-      <c r="H8" s="67">
-        <f>'Revenue Forecast'!BL35</f>
-        <v/>
-      </c>
-      <c r="J8" s="20" t="inlineStr">
-        <is>
-          <t>the reason the plan could not sell more in the last month of the year</t>
-        </is>
+          <t>Build capacity used</t>
+        </is>
+      </c>
+      <c r="D8" s="48">
+        <f>'Revenue Forecast'!BN35</f>
+        <v/>
+      </c>
+      <c r="E8" s="48">
+        <f>'Revenue Forecast'!BO35</f>
+        <v/>
+      </c>
+      <c r="F8" s="48">
+        <f>'Revenue Forecast'!BP35</f>
+        <v/>
+      </c>
+      <c r="G8" s="48">
+        <f>'Revenue Forecast'!BQ35</f>
+        <v/>
+      </c>
+      <c r="H8" s="48">
+        <f>'Revenue Forecast'!BR35</f>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Build capacity used</t>
-        </is>
-      </c>
-      <c r="D9" s="48">
-        <f>'Revenue Forecast'!BN36</f>
-        <v/>
-      </c>
-      <c r="E9" s="48">
-        <f>'Revenue Forecast'!BO36</f>
-        <v/>
-      </c>
-      <c r="F9" s="48">
-        <f>'Revenue Forecast'!BP36</f>
-        <v/>
-      </c>
-      <c r="G9" s="48">
-        <f>'Revenue Forecast'!BQ36</f>
-        <v/>
-      </c>
-      <c r="H9" s="48">
-        <f>'Revenue Forecast'!BR36</f>
+          <t>Installer partners at year end</t>
+        </is>
+      </c>
+      <c r="D9" s="62">
+        <f>'Revenue Forecast'!BN20</f>
+        <v/>
+      </c>
+      <c r="E9" s="62">
+        <f>'Revenue Forecast'!BO20</f>
+        <v/>
+      </c>
+      <c r="F9" s="62">
+        <f>'Revenue Forecast'!BP20</f>
+        <v/>
+      </c>
+      <c r="G9" s="62">
+        <f>'Revenue Forecast'!BQ20</f>
+        <v/>
+      </c>
+      <c r="H9" s="62">
+        <f>'Revenue Forecast'!BR20</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Installer partners at year end</t>
-        </is>
-      </c>
-      <c r="D10" s="62">
-        <f>'Revenue Forecast'!BN20</f>
-        <v/>
-      </c>
-      <c r="E10" s="62">
-        <f>'Revenue Forecast'!BO20</f>
-        <v/>
-      </c>
-      <c r="F10" s="62">
-        <f>'Revenue Forecast'!BP20</f>
-        <v/>
-      </c>
-      <c r="G10" s="62">
-        <f>'Revenue Forecast'!BQ20</f>
-        <v/>
-      </c>
-      <c r="H10" s="62">
-        <f>'Revenue Forecast'!BR20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="9" t="inlineStr">
-        <is>
           <t>Marketing cost per unit sold</t>
         </is>
       </c>
-      <c r="D11" s="43">
+      <c r="D10" s="43">
         <f>'Revenue Forecast'!BN12</f>
         <v/>
       </c>
-      <c r="E11" s="43">
+      <c r="E10" s="43">
         <f>'Revenue Forecast'!BO12</f>
         <v/>
       </c>
-      <c r="F11" s="43">
+      <c r="F10" s="43">
         <f>'Revenue Forecast'!BP12</f>
         <v/>
       </c>
-      <c r="G11" s="43">
+      <c r="G10" s="43">
         <f>'Revenue Forecast'!BQ12</f>
         <v/>
       </c>
-      <c r="H11" s="43">
+      <c r="H10" s="43">
         <f>'Revenue Forecast'!BR12</f>
         <v/>
       </c>
@@ -48309,7 +47997,7 @@
           <t>Balance sheet check, worst month across the whole model</t>
         </is>
       </c>
-      <c r="D34" s="72">
+      <c r="D34" s="70">
         <f>MAX(ABS(MIN('Financial Statements'!$E$58:$BL$58)),ABS(MAX('Financial Statements'!$E$58:$BL$58)))</f>
         <v/>
       </c>
@@ -48356,7 +48044,7 @@
           <t>The month it happens</t>
         </is>
       </c>
-      <c r="D38" s="73">
+      <c r="D38" s="71">
         <f>INDEX('Financial Statements'!$E$3:$BL$3,MATCH(D37,'Financial Statements'!$N$40:$BL$40,0)+9)</f>
         <v/>
       </c>
@@ -48507,7 +48195,7 @@
           <t>Share of the raise the plan actually uses</t>
         </is>
       </c>
-      <c r="D52" s="74">
+      <c r="D52" s="72">
         <f>IFERROR(D51/SUM('Financial Statements'!N35:BL35),0)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Tarnoc v2: BOM tier basis 2 no longer drops a tier in the final year (next year taken as at least this year)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Tarnoc_v2_2026-09-01.xlsx
+++ b/models/Tarnoc_v2_2026-09-01.xlsx
@@ -29366,243 +29366,243 @@
         </is>
       </c>
       <c r="E7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(E$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(E$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),E6)</f>
         <v/>
       </c>
       <c r="F7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(F$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(F$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),F6)</f>
         <v/>
       </c>
       <c r="G7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(G$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(G$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),G6)</f>
         <v/>
       </c>
       <c r="H7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(H$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(H$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),H6)</f>
         <v/>
       </c>
       <c r="I7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(I$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(I$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),I6)</f>
         <v/>
       </c>
       <c r="J7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(J$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(J$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),J6)</f>
         <v/>
       </c>
       <c r="K7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(K$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(K$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),K6)</f>
         <v/>
       </c>
       <c r="L7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(L$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(L$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),L6)</f>
         <v/>
       </c>
       <c r="M7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(M$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(M$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),M6)</f>
         <v/>
       </c>
       <c r="N7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(N$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(N$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),N6)</f>
         <v/>
       </c>
       <c r="O7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(O$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(O$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),O6)</f>
         <v/>
       </c>
       <c r="P7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(P$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(P$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),P6)</f>
         <v/>
       </c>
       <c r="Q7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(Q$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(Q$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),Q6)</f>
         <v/>
       </c>
       <c r="R7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(R$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(R$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),R6)</f>
         <v/>
       </c>
       <c r="S7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(S$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(S$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),S6)</f>
         <v/>
       </c>
       <c r="T7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(T$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(T$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),T6)</f>
         <v/>
       </c>
       <c r="U7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(U$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(U$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),U6)</f>
         <v/>
       </c>
       <c r="V7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(V$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(V$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),V6)</f>
         <v/>
       </c>
       <c r="W7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(W$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(W$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),W6)</f>
         <v/>
       </c>
       <c r="X7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(X$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(X$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),X6)</f>
         <v/>
       </c>
       <c r="Y7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(Y$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(Y$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),Y6)</f>
         <v/>
       </c>
       <c r="Z7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(Z$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(Z$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),Z6)</f>
         <v/>
       </c>
       <c r="AA7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AA$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AA$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AA6)</f>
         <v/>
       </c>
       <c r="AB7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AB$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AB$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AB6)</f>
         <v/>
       </c>
       <c r="AC7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AC$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AC$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AC6)</f>
         <v/>
       </c>
       <c r="AD7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AD$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AD$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AD6)</f>
         <v/>
       </c>
       <c r="AE7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AE$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AE$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AE6)</f>
         <v/>
       </c>
       <c r="AF7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AF$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AF$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AF6)</f>
         <v/>
       </c>
       <c r="AG7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AG$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AG$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AG6)</f>
         <v/>
       </c>
       <c r="AH7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AH$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AH$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AH6)</f>
         <v/>
       </c>
       <c r="AI7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AI$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AI$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AI6)</f>
         <v/>
       </c>
       <c r="AJ7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AJ$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AJ$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AJ6)</f>
         <v/>
       </c>
       <c r="AK7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AK$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AK$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AK6)</f>
         <v/>
       </c>
       <c r="AL7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AL$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AL$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AL6)</f>
         <v/>
       </c>
       <c r="AM7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AM$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AM$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AM6)</f>
         <v/>
       </c>
       <c r="AN7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AN$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AN$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AN6)</f>
         <v/>
       </c>
       <c r="AO7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AO$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AO$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AO6)</f>
         <v/>
       </c>
       <c r="AP7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AP$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AP$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AP6)</f>
         <v/>
       </c>
       <c r="AQ7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AQ$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AQ$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AQ6)</f>
         <v/>
       </c>
       <c r="AR7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AR$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AR$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AR6)</f>
         <v/>
       </c>
       <c r="AS7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AS$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AS$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AS6)</f>
         <v/>
       </c>
       <c r="AT7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AT$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AT$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AT6)</f>
         <v/>
       </c>
       <c r="AU7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AU$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AU$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AU6)</f>
         <v/>
       </c>
       <c r="AV7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AV$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AV$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AV6)</f>
         <v/>
       </c>
       <c r="AW7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AW$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AW$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AW6)</f>
         <v/>
       </c>
       <c r="AX7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AX$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AX$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AX6)</f>
         <v/>
       </c>
       <c r="AY7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AY$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AY$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AY6)</f>
         <v/>
       </c>
       <c r="AZ7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(AZ$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(AZ$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),AZ6)</f>
         <v/>
       </c>
       <c r="BA7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(BA$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(BA$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),BA6)</f>
         <v/>
       </c>
       <c r="BB7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(BB$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(BB$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),BB6)</f>
         <v/>
       </c>
       <c r="BC7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(BC$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(BC$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),BC6)</f>
         <v/>
       </c>
       <c r="BD7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(BD$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(BD$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),BD6)</f>
         <v/>
       </c>
       <c r="BE7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(BE$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(BE$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),BE6)</f>
         <v/>
       </c>
       <c r="BF7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(BF$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(BF$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),BF6)</f>
         <v/>
       </c>
       <c r="BG7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(BG$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(BG$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),BG6)</f>
         <v/>
       </c>
       <c r="BH7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(BH$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(BH$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),BH6)</f>
         <v/>
       </c>
       <c r="BI7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(BI$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(BI$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),BI6)</f>
         <v/>
       </c>
       <c r="BJ7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(BJ$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(BJ$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),BJ6)</f>
         <v/>
       </c>
       <c r="BK7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(BK$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(BK$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),BK6)</f>
         <v/>
       </c>
       <c r="BL7" s="54">
-        <f>IFERROR(HLOOKUP(YEAR(BL$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),0)</f>
+        <f>IFERROR(HLOOKUP(YEAR(BL$3)+1,'Revenue Forecast'!$BN$3:$BR$34,32,FALSE),BL6)</f>
         <v/>
       </c>
       <c r="BN7" s="55">
@@ -29627,7 +29627,7 @@
       </c>
       <c r="BT7" s="20" t="inlineStr">
         <is>
-          <t>only used when the tier basis switch is set to 2</t>
+          <t>only used when the tier basis switch is set to 2; beyond the horizon, next year is taken as at least this year</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tarnoc v2: clearer label and note for the field engineer sizing ratio
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Tarnoc_v2_2026-09-01.xlsx
+++ b/models/Tarnoc_v2_2026-09-01.xlsx
@@ -4017,12 +4017,12 @@
     <row r="122">
       <c r="B122" s="9" t="inlineStr">
         <is>
-          <t>Units on a service contract per field engineer</t>
+          <t>Boilers one field engineer can look after</t>
         </is>
       </c>
       <c r="C122" s="18" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>boilers</t>
         </is>
       </c>
       <c r="D122" s="29" t="n">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="J122" s="20" t="inlineStr">
         <is>
-          <t>one visit per contract per year, so about three and a half visits per engineer per working day</t>
+          <t>sizes the field service team: boilers on a service contract divided by this number = engineers to hire. Each boiler gets one visit a year, an engineer does three to four a day</t>
         </is>
       </c>
     </row>
@@ -44863,7 +44863,7 @@
       </c>
       <c r="BT19" s="20" t="inlineStr">
         <is>
-          <t>salaried staff: one engineer per 750 units on a service contract</t>
+          <t>salaried staff: boilers on a service contract divided by the boilers one engineer can look after</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tarnoc v2: TTK/Combi+ mix 25/75, no inventory in either case, aggressive R&D hiring +2 a year
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Tarnoc_v2_2026-09-01.xlsx
+++ b/models/Tarnoc_v2_2026-09-01.xlsx
@@ -1742,7 +1742,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="29" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F21" s="30">
         <f>IF(Assumptions!$E$5=2,E21,D21)</f>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="J21" s="20" t="inlineStr">
         <is>
-          <t>the aggressive case carries stock, the base case does not</t>
+          <t>the assembly partner holds the stock; nothing sits on our balance sheet</t>
         </is>
       </c>
     </row>
@@ -1895,10 +1895,10 @@
         </is>
       </c>
       <c r="D28" s="25" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="E28" s="25" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="F28" s="26">
         <f>IF(Assumptions!$E$5=2,E28,D28)</f>
@@ -3507,16 +3507,16 @@
         <v>0</v>
       </c>
       <c r="E101" s="29" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F101" s="29" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G101" s="29" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H101" s="29" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="102">

</xml_diff>

<commit_message>
Tarnoc v2: TTK share back to 20%; aggressive in-house line 1 producing from Nov-2027 (paid Nov-2026)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Tarnoc_v2_2026-09-01.xlsx
+++ b/models/Tarnoc_v2_2026-09-01.xlsx
@@ -1895,10 +1895,10 @@
         </is>
       </c>
       <c r="D28" s="25" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="E28" s="25" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="F28" s="26">
         <f>IF(Assumptions!$E$5=2,E28,D28)</f>
@@ -3093,7 +3093,7 @@
         <v>49310</v>
       </c>
       <c r="E82" s="27" t="n">
-        <v>46935</v>
+        <v>46692</v>
       </c>
       <c r="F82" s="28">
         <f>IF(Assumptions!$E$5=2,E82,D82)</f>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="J82" s="20" t="inlineStr">
         <is>
-          <t>set well past the horizon to mean never, so the capex lead time cannot pull spend in</t>
+          <t>base: set well past the horizon to mean never. Aggressive: paid for in November 2026, the first month after the raise lands</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tarnoc v2: the turbineketel is a turbine heat pump, not a boiler; labels and research framing corrected
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Tarnoc_v2_2026-09-01.xlsx
+++ b/models/Tarnoc_v2_2026-09-01.xlsx
@@ -2967,7 +2967,7 @@
     <row r="77">
       <c r="B77" s="9" t="inlineStr">
         <is>
-          <t>Installer partner commission, share of boiler price</t>
+          <t>Installer partner commission, share of unit price</t>
         </is>
       </c>
       <c r="C77" s="18" t="inlineStr">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="J77" s="20" t="inlineStr">
         <is>
-          <t>paid on every unit sold through the channel, on the boiler price only, not on installation or upsell</t>
+          <t>paid on every unit sold through the channel, on the turbineketel or Combi+ system price only, not on installation, upsell or service</t>
         </is>
       </c>
     </row>
@@ -3786,12 +3786,12 @@
     <row r="113">
       <c r="B113" s="9" t="inlineStr">
         <is>
-          <t>Boilers one field engineer can look after</t>
+          <t>Installed units one field engineer can look after</t>
         </is>
       </c>
       <c r="C113" s="18" t="inlineStr">
         <is>
-          <t>boilers</t>
+          <t>units</t>
         </is>
       </c>
       <c r="D113" s="29" t="n">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="J113" s="20" t="inlineStr">
         <is>
-          <t>sizes the field service team: boilers on a service contract divided by this number = engineers to hire. Each boiler gets one visit a year, an engineer does three to four a day</t>
+          <t>sizes the field service team: units on a service contract divided by this number = engineers to hire. Each unit gets one visit a year, an engineer does three to four a day</t>
         </is>
       </c>
     </row>
@@ -31945,7 +31945,7 @@
       </c>
       <c r="BT18" s="20" t="inlineStr">
         <is>
-          <t>boiler revenue on the channel share of units, times the commission rate</t>
+          <t>turbineketel and Combi+ revenue on the channel share of units, times the commission rate</t>
         </is>
       </c>
     </row>
@@ -44300,7 +44300,7 @@
       </c>
       <c r="BT18" s="20" t="inlineStr">
         <is>
-          <t>salaried staff: boilers on a service contract divided by the boilers one engineer can look after</t>
+          <t>salaried staff: installed units on a service contract divided by the units one engineer can look after</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tarnoc v2: formula review fixes: annual ratios recomputed from totals, opening cash by year, dashboard follows the raise date, revenue per person, receivables exclude the subsidy, overheads inflate, labels; review report added
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Tarnoc_v2_2026-09-01.xlsx
+++ b/models/Tarnoc_v2_2026-09-01.xlsx
@@ -1524,7 +1524,7 @@
     <row r="12">
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Interest on the working capital loan</t>
+          <t>Interest on the convertible loan</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
@@ -5987,23 +5987,23 @@
         <v/>
       </c>
       <c r="BN9" s="49">
-        <f>IFERROR(AVERAGE(E9:P9),0)</f>
+        <f>IFERROR(BN8/BN6,0)</f>
         <v/>
       </c>
       <c r="BO9" s="49">
-        <f>IFERROR(AVERAGE(Q9:AB9),0)</f>
+        <f>IFERROR(BO8/BO6,0)</f>
         <v/>
       </c>
       <c r="BP9" s="49">
-        <f>IFERROR(AVERAGE(AC9:AN9),0)</f>
+        <f>IFERROR(BP8/BP6,0)</f>
         <v/>
       </c>
       <c r="BQ9" s="49">
-        <f>IFERROR(AVERAGE(AO9:AZ9),0)</f>
+        <f>IFERROR(BQ8/BQ6,0)</f>
         <v/>
       </c>
       <c r="BR9" s="49">
-        <f>IFERROR(AVERAGE(BA9:BL9),0)</f>
+        <f>IFERROR(BR8/BR6,0)</f>
         <v/>
       </c>
     </row>
@@ -7622,23 +7622,23 @@
         <v/>
       </c>
       <c r="BN17" s="49">
-        <f>IFERROR(AVERAGE(E17:P17),0)</f>
+        <f>IFERROR(BN16/BN6,0)</f>
         <v/>
       </c>
       <c r="BO17" s="49">
-        <f>IFERROR(AVERAGE(Q17:AB17),0)</f>
+        <f>IFERROR(BO16/BO6,0)</f>
         <v/>
       </c>
       <c r="BP17" s="49">
-        <f>IFERROR(AVERAGE(AC17:AN17),0)</f>
+        <f>IFERROR(BP16/BP6,0)</f>
         <v/>
       </c>
       <c r="BQ17" s="49">
-        <f>IFERROR(AVERAGE(AO17:AZ17),0)</f>
+        <f>IFERROR(BQ16/BQ6,0)</f>
         <v/>
       </c>
       <c r="BR17" s="49">
-        <f>IFERROR(AVERAGE(BA17:BL17),0)</f>
+        <f>IFERROR(BR16/BR6,0)</f>
         <v/>
       </c>
     </row>
@@ -9267,23 +9267,23 @@
         <v/>
       </c>
       <c r="BN24" s="49">
-        <f>IFERROR(AVERAGE(E24:P24),0)</f>
+        <f>IFERROR(BN23/BN6,0)</f>
         <v/>
       </c>
       <c r="BO24" s="49">
-        <f>IFERROR(AVERAGE(Q24:AB24),0)</f>
+        <f>IFERROR(BO23/BO6,0)</f>
         <v/>
       </c>
       <c r="BP24" s="49">
-        <f>IFERROR(AVERAGE(AC24:AN24),0)</f>
+        <f>IFERROR(BP23/BP6,0)</f>
         <v/>
       </c>
       <c r="BQ24" s="49">
-        <f>IFERROR(AVERAGE(AO24:AZ24),0)</f>
+        <f>IFERROR(BQ23/BQ6,0)</f>
         <v/>
       </c>
       <c r="BR24" s="49">
-        <f>IFERROR(AVERAGE(BA24:BL24),0)</f>
+        <f>IFERROR(BR23/BR6,0)</f>
         <v/>
       </c>
     </row>
@@ -12884,23 +12884,23 @@
         <v/>
       </c>
       <c r="BN39" s="44">
-        <f>P39</f>
+        <f>E39</f>
         <v/>
       </c>
       <c r="BO39" s="44">
-        <f>AB39</f>
+        <f>Q39</f>
         <v/>
       </c>
       <c r="BP39" s="44">
-        <f>AN39</f>
+        <f>AC39</f>
         <v/>
       </c>
       <c r="BQ39" s="44">
-        <f>AZ39</f>
+        <f>AO39</f>
         <v/>
       </c>
       <c r="BR39" s="44">
-        <f>BL39</f>
+        <f>BA39</f>
         <v/>
       </c>
     </row>
@@ -13536,243 +13536,243 @@
         </is>
       </c>
       <c r="E44" s="43">
-        <f>Assumptions!$F$19/30*E6</f>
+        <f>Assumptions!$F$19/30*(E6-'Revenue Forecast'!E49)</f>
         <v/>
       </c>
       <c r="F44" s="43">
-        <f>Assumptions!$F$19/30*F6</f>
+        <f>Assumptions!$F$19/30*(F6-'Revenue Forecast'!F49)</f>
         <v/>
       </c>
       <c r="G44" s="43">
-        <f>Assumptions!$F$19/30*G6</f>
+        <f>Assumptions!$F$19/30*(G6-'Revenue Forecast'!G49)</f>
         <v/>
       </c>
       <c r="H44" s="43">
-        <f>Assumptions!$F$19/30*H6</f>
+        <f>Assumptions!$F$19/30*(H6-'Revenue Forecast'!H49)</f>
         <v/>
       </c>
       <c r="I44" s="43">
-        <f>Assumptions!$F$19/30*I6</f>
+        <f>Assumptions!$F$19/30*(I6-'Revenue Forecast'!I49)</f>
         <v/>
       </c>
       <c r="J44" s="43">
-        <f>Assumptions!$F$19/30*J6</f>
+        <f>Assumptions!$F$19/30*(J6-'Revenue Forecast'!J49)</f>
         <v/>
       </c>
       <c r="K44" s="43">
-        <f>Assumptions!$F$19/30*K6</f>
+        <f>Assumptions!$F$19/30*(K6-'Revenue Forecast'!K49)</f>
         <v/>
       </c>
       <c r="L44" s="43">
-        <f>Assumptions!$F$19/30*L6</f>
+        <f>Assumptions!$F$19/30*(L6-'Revenue Forecast'!L49)</f>
         <v/>
       </c>
       <c r="M44" s="43">
-        <f>Assumptions!$F$19/30*M6</f>
+        <f>Assumptions!$F$19/30*(M6-'Revenue Forecast'!M49)</f>
         <v/>
       </c>
       <c r="N44" s="43">
-        <f>Assumptions!$F$19/30*N6</f>
+        <f>Assumptions!$F$19/30*(N6-'Revenue Forecast'!N49)</f>
         <v/>
       </c>
       <c r="O44" s="43">
-        <f>Assumptions!$F$19/30*O6</f>
+        <f>Assumptions!$F$19/30*(O6-'Revenue Forecast'!O49)</f>
         <v/>
       </c>
       <c r="P44" s="43">
-        <f>Assumptions!$F$19/30*P6</f>
+        <f>Assumptions!$F$19/30*(P6-'Revenue Forecast'!P49)</f>
         <v/>
       </c>
       <c r="Q44" s="43">
-        <f>Assumptions!$F$19/30*Q6</f>
+        <f>Assumptions!$F$19/30*(Q6-'Revenue Forecast'!Q49)</f>
         <v/>
       </c>
       <c r="R44" s="43">
-        <f>Assumptions!$F$19/30*R6</f>
+        <f>Assumptions!$F$19/30*(R6-'Revenue Forecast'!R49)</f>
         <v/>
       </c>
       <c r="S44" s="43">
-        <f>Assumptions!$F$19/30*S6</f>
+        <f>Assumptions!$F$19/30*(S6-'Revenue Forecast'!S49)</f>
         <v/>
       </c>
       <c r="T44" s="43">
-        <f>Assumptions!$F$19/30*T6</f>
+        <f>Assumptions!$F$19/30*(T6-'Revenue Forecast'!T49)</f>
         <v/>
       </c>
       <c r="U44" s="43">
-        <f>Assumptions!$F$19/30*U6</f>
+        <f>Assumptions!$F$19/30*(U6-'Revenue Forecast'!U49)</f>
         <v/>
       </c>
       <c r="V44" s="43">
-        <f>Assumptions!$F$19/30*V6</f>
+        <f>Assumptions!$F$19/30*(V6-'Revenue Forecast'!V49)</f>
         <v/>
       </c>
       <c r="W44" s="43">
-        <f>Assumptions!$F$19/30*W6</f>
+        <f>Assumptions!$F$19/30*(W6-'Revenue Forecast'!W49)</f>
         <v/>
       </c>
       <c r="X44" s="43">
-        <f>Assumptions!$F$19/30*X6</f>
+        <f>Assumptions!$F$19/30*(X6-'Revenue Forecast'!X49)</f>
         <v/>
       </c>
       <c r="Y44" s="43">
-        <f>Assumptions!$F$19/30*Y6</f>
+        <f>Assumptions!$F$19/30*(Y6-'Revenue Forecast'!Y49)</f>
         <v/>
       </c>
       <c r="Z44" s="43">
-        <f>Assumptions!$F$19/30*Z6</f>
+        <f>Assumptions!$F$19/30*(Z6-'Revenue Forecast'!Z49)</f>
         <v/>
       </c>
       <c r="AA44" s="43">
-        <f>Assumptions!$F$19/30*AA6</f>
+        <f>Assumptions!$F$19/30*(AA6-'Revenue Forecast'!AA49)</f>
         <v/>
       </c>
       <c r="AB44" s="43">
-        <f>Assumptions!$F$19/30*AB6</f>
+        <f>Assumptions!$F$19/30*(AB6-'Revenue Forecast'!AB49)</f>
         <v/>
       </c>
       <c r="AC44" s="43">
-        <f>Assumptions!$F$19/30*AC6</f>
+        <f>Assumptions!$F$19/30*(AC6-'Revenue Forecast'!AC49)</f>
         <v/>
       </c>
       <c r="AD44" s="43">
-        <f>Assumptions!$F$19/30*AD6</f>
+        <f>Assumptions!$F$19/30*(AD6-'Revenue Forecast'!AD49)</f>
         <v/>
       </c>
       <c r="AE44" s="43">
-        <f>Assumptions!$F$19/30*AE6</f>
+        <f>Assumptions!$F$19/30*(AE6-'Revenue Forecast'!AE49)</f>
         <v/>
       </c>
       <c r="AF44" s="43">
-        <f>Assumptions!$F$19/30*AF6</f>
+        <f>Assumptions!$F$19/30*(AF6-'Revenue Forecast'!AF49)</f>
         <v/>
       </c>
       <c r="AG44" s="43">
-        <f>Assumptions!$F$19/30*AG6</f>
+        <f>Assumptions!$F$19/30*(AG6-'Revenue Forecast'!AG49)</f>
         <v/>
       </c>
       <c r="AH44" s="43">
-        <f>Assumptions!$F$19/30*AH6</f>
+        <f>Assumptions!$F$19/30*(AH6-'Revenue Forecast'!AH49)</f>
         <v/>
       </c>
       <c r="AI44" s="43">
-        <f>Assumptions!$F$19/30*AI6</f>
+        <f>Assumptions!$F$19/30*(AI6-'Revenue Forecast'!AI49)</f>
         <v/>
       </c>
       <c r="AJ44" s="43">
-        <f>Assumptions!$F$19/30*AJ6</f>
+        <f>Assumptions!$F$19/30*(AJ6-'Revenue Forecast'!AJ49)</f>
         <v/>
       </c>
       <c r="AK44" s="43">
-        <f>Assumptions!$F$19/30*AK6</f>
+        <f>Assumptions!$F$19/30*(AK6-'Revenue Forecast'!AK49)</f>
         <v/>
       </c>
       <c r="AL44" s="43">
-        <f>Assumptions!$F$19/30*AL6</f>
+        <f>Assumptions!$F$19/30*(AL6-'Revenue Forecast'!AL49)</f>
         <v/>
       </c>
       <c r="AM44" s="43">
-        <f>Assumptions!$F$19/30*AM6</f>
+        <f>Assumptions!$F$19/30*(AM6-'Revenue Forecast'!AM49)</f>
         <v/>
       </c>
       <c r="AN44" s="43">
-        <f>Assumptions!$F$19/30*AN6</f>
+        <f>Assumptions!$F$19/30*(AN6-'Revenue Forecast'!AN49)</f>
         <v/>
       </c>
       <c r="AO44" s="43">
-        <f>Assumptions!$F$19/30*AO6</f>
+        <f>Assumptions!$F$19/30*(AO6-'Revenue Forecast'!AO49)</f>
         <v/>
       </c>
       <c r="AP44" s="43">
-        <f>Assumptions!$F$19/30*AP6</f>
+        <f>Assumptions!$F$19/30*(AP6-'Revenue Forecast'!AP49)</f>
         <v/>
       </c>
       <c r="AQ44" s="43">
-        <f>Assumptions!$F$19/30*AQ6</f>
+        <f>Assumptions!$F$19/30*(AQ6-'Revenue Forecast'!AQ49)</f>
         <v/>
       </c>
       <c r="AR44" s="43">
-        <f>Assumptions!$F$19/30*AR6</f>
+        <f>Assumptions!$F$19/30*(AR6-'Revenue Forecast'!AR49)</f>
         <v/>
       </c>
       <c r="AS44" s="43">
-        <f>Assumptions!$F$19/30*AS6</f>
+        <f>Assumptions!$F$19/30*(AS6-'Revenue Forecast'!AS49)</f>
         <v/>
       </c>
       <c r="AT44" s="43">
-        <f>Assumptions!$F$19/30*AT6</f>
+        <f>Assumptions!$F$19/30*(AT6-'Revenue Forecast'!AT49)</f>
         <v/>
       </c>
       <c r="AU44" s="43">
-        <f>Assumptions!$F$19/30*AU6</f>
+        <f>Assumptions!$F$19/30*(AU6-'Revenue Forecast'!AU49)</f>
         <v/>
       </c>
       <c r="AV44" s="43">
-        <f>Assumptions!$F$19/30*AV6</f>
+        <f>Assumptions!$F$19/30*(AV6-'Revenue Forecast'!AV49)</f>
         <v/>
       </c>
       <c r="AW44" s="43">
-        <f>Assumptions!$F$19/30*AW6</f>
+        <f>Assumptions!$F$19/30*(AW6-'Revenue Forecast'!AW49)</f>
         <v/>
       </c>
       <c r="AX44" s="43">
-        <f>Assumptions!$F$19/30*AX6</f>
+        <f>Assumptions!$F$19/30*(AX6-'Revenue Forecast'!AX49)</f>
         <v/>
       </c>
       <c r="AY44" s="43">
-        <f>Assumptions!$F$19/30*AY6</f>
+        <f>Assumptions!$F$19/30*(AY6-'Revenue Forecast'!AY49)</f>
         <v/>
       </c>
       <c r="AZ44" s="43">
-        <f>Assumptions!$F$19/30*AZ6</f>
+        <f>Assumptions!$F$19/30*(AZ6-'Revenue Forecast'!AZ49)</f>
         <v/>
       </c>
       <c r="BA44" s="43">
-        <f>Assumptions!$F$19/30*BA6</f>
+        <f>Assumptions!$F$19/30*(BA6-'Revenue Forecast'!BA49)</f>
         <v/>
       </c>
       <c r="BB44" s="43">
-        <f>Assumptions!$F$19/30*BB6</f>
+        <f>Assumptions!$F$19/30*(BB6-'Revenue Forecast'!BB49)</f>
         <v/>
       </c>
       <c r="BC44" s="43">
-        <f>Assumptions!$F$19/30*BC6</f>
+        <f>Assumptions!$F$19/30*(BC6-'Revenue Forecast'!BC49)</f>
         <v/>
       </c>
       <c r="BD44" s="43">
-        <f>Assumptions!$F$19/30*BD6</f>
+        <f>Assumptions!$F$19/30*(BD6-'Revenue Forecast'!BD49)</f>
         <v/>
       </c>
       <c r="BE44" s="43">
-        <f>Assumptions!$F$19/30*BE6</f>
+        <f>Assumptions!$F$19/30*(BE6-'Revenue Forecast'!BE49)</f>
         <v/>
       </c>
       <c r="BF44" s="43">
-        <f>Assumptions!$F$19/30*BF6</f>
+        <f>Assumptions!$F$19/30*(BF6-'Revenue Forecast'!BF49)</f>
         <v/>
       </c>
       <c r="BG44" s="43">
-        <f>Assumptions!$F$19/30*BG6</f>
+        <f>Assumptions!$F$19/30*(BG6-'Revenue Forecast'!BG49)</f>
         <v/>
       </c>
       <c r="BH44" s="43">
-        <f>Assumptions!$F$19/30*BH6</f>
+        <f>Assumptions!$F$19/30*(BH6-'Revenue Forecast'!BH49)</f>
         <v/>
       </c>
       <c r="BI44" s="43">
-        <f>Assumptions!$F$19/30*BI6</f>
+        <f>Assumptions!$F$19/30*(BI6-'Revenue Forecast'!BI49)</f>
         <v/>
       </c>
       <c r="BJ44" s="43">
-        <f>Assumptions!$F$19/30*BJ6</f>
+        <f>Assumptions!$F$19/30*(BJ6-'Revenue Forecast'!BJ49)</f>
         <v/>
       </c>
       <c r="BK44" s="43">
-        <f>Assumptions!$F$19/30*BK6</f>
+        <f>Assumptions!$F$19/30*(BK6-'Revenue Forecast'!BK49)</f>
         <v/>
       </c>
       <c r="BL44" s="43">
-        <f>Assumptions!$F$19/30*BL6</f>
+        <f>Assumptions!$F$19/30*(BL6-'Revenue Forecast'!BL49)</f>
         <v/>
       </c>
       <c r="BN44" s="44">
@@ -13794,6 +13794,11 @@
       <c r="BR44" s="44">
         <f>BL44</f>
         <v/>
+      </c>
+      <c r="BT44" s="20" t="inlineStr">
+        <is>
+          <t>on trading revenue only; the subsidy is a cash receipt, not an invoice</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -23418,23 +23423,23 @@
         <v/>
       </c>
       <c r="BN24" s="63">
-        <f>IFERROR(AVERAGE(E24:P24),0)</f>
+        <f>IFERROR(BN34/BN22,0)</f>
         <v/>
       </c>
       <c r="BO24" s="63">
-        <f>IFERROR(AVERAGE(Q24:AB24),0)</f>
+        <f>IFERROR(BO34/BO22,0)</f>
         <v/>
       </c>
       <c r="BP24" s="63">
-        <f>IFERROR(AVERAGE(AC24:AN24),0)</f>
+        <f>IFERROR(BP34/BP22,0)</f>
         <v/>
       </c>
       <c r="BQ24" s="63">
-        <f>IFERROR(AVERAGE(AO24:AZ24),0)</f>
+        <f>IFERROR(BQ34/BQ22,0)</f>
         <v/>
       </c>
       <c r="BR24" s="63">
-        <f>IFERROR(AVERAGE(BA24:BL24),0)</f>
+        <f>IFERROR(BR34/BR22,0)</f>
         <v/>
       </c>
     </row>
@@ -25215,23 +25220,23 @@
         <v/>
       </c>
       <c r="BN35" s="63">
-        <f>IFERROR(AVERAGE(E35:P35),0)</f>
+        <f>IFERROR(BN34/BN31,0)</f>
         <v/>
       </c>
       <c r="BO35" s="63">
-        <f>IFERROR(AVERAGE(Q35:AB35),0)</f>
+        <f>IFERROR(BO34/BO31,0)</f>
         <v/>
       </c>
       <c r="BP35" s="63">
-        <f>IFERROR(AVERAGE(AC35:AN35),0)</f>
+        <f>IFERROR(BP34/BP31,0)</f>
         <v/>
       </c>
       <c r="BQ35" s="63">
-        <f>IFERROR(AVERAGE(AO35:AZ35),0)</f>
+        <f>IFERROR(BQ34/BQ31,0)</f>
         <v/>
       </c>
       <c r="BR35" s="63">
-        <f>IFERROR(AVERAGE(BA35:BL35),0)</f>
+        <f>IFERROR(BR34/BR31,0)</f>
         <v/>
       </c>
     </row>
@@ -28377,23 +28382,23 @@
         <v/>
       </c>
       <c r="BN51" s="66">
-        <f>IFERROR(AVERAGE(E51:P51),0)</f>
+        <f>IFERROR((BN50-BN49)/BN34,0)</f>
         <v/>
       </c>
       <c r="BO51" s="66">
-        <f>IFERROR(AVERAGE(Q51:AB51),0)</f>
+        <f>IFERROR((BO50-BO49)/BO34,0)</f>
         <v/>
       </c>
       <c r="BP51" s="66">
-        <f>IFERROR(AVERAGE(AC51:AN51),0)</f>
+        <f>IFERROR((BP50-BP49)/BP34,0)</f>
         <v/>
       </c>
       <c r="BQ51" s="66">
-        <f>IFERROR(AVERAGE(AO51:AZ51),0)</f>
+        <f>IFERROR((BQ50-BQ49)/BQ34,0)</f>
         <v/>
       </c>
       <c r="BR51" s="66">
-        <f>IFERROR(AVERAGE(BA51:BL51),0)</f>
+        <f>IFERROR((BR50-BR49)/BR34,0)</f>
         <v/>
       </c>
     </row>
@@ -32476,23 +32481,23 @@
         <v/>
       </c>
       <c r="BN21" s="66">
-        <f>IFERROR(AVERAGE(E21:P21),0)</f>
+        <f>IFERROR(('Revenue Forecast'!BN50-BN19)/'Revenue Forecast'!BN34,0)</f>
         <v/>
       </c>
       <c r="BO21" s="66">
-        <f>IFERROR(AVERAGE(Q21:AB21),0)</f>
+        <f>IFERROR(('Revenue Forecast'!BO50-BO19)/'Revenue Forecast'!BO34,0)</f>
         <v/>
       </c>
       <c r="BP21" s="66">
-        <f>IFERROR(AVERAGE(AC21:AN21),0)</f>
+        <f>IFERROR(('Revenue Forecast'!BP50-BP19)/'Revenue Forecast'!BP34,0)</f>
         <v/>
       </c>
       <c r="BQ21" s="66">
-        <f>IFERROR(AVERAGE(AO21:AZ21),0)</f>
+        <f>IFERROR(('Revenue Forecast'!BQ50-BQ19)/'Revenue Forecast'!BQ34,0)</f>
         <v/>
       </c>
       <c r="BR21" s="66">
-        <f>IFERROR(AVERAGE(BA21:BL21),0)</f>
+        <f>IFERROR(('Revenue Forecast'!BR50-BR19)/'Revenue Forecast'!BR34,0)</f>
         <v/>
       </c>
     </row>
@@ -34403,243 +34408,243 @@
         </is>
       </c>
       <c r="E13" s="43">
-        <f>'Revenue Forecast'!E19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!E19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(E$3)-2026)</f>
         <v/>
       </c>
       <c r="F13" s="43">
-        <f>'Revenue Forecast'!F19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!F19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(F$3)-2026)</f>
         <v/>
       </c>
       <c r="G13" s="43">
-        <f>'Revenue Forecast'!G19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!G19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(G$3)-2026)</f>
         <v/>
       </c>
       <c r="H13" s="43">
-        <f>'Revenue Forecast'!H19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!H19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(H$3)-2026)</f>
         <v/>
       </c>
       <c r="I13" s="43">
-        <f>'Revenue Forecast'!I19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!I19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(I$3)-2026)</f>
         <v/>
       </c>
       <c r="J13" s="43">
-        <f>'Revenue Forecast'!J19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!J19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(J$3)-2026)</f>
         <v/>
       </c>
       <c r="K13" s="43">
-        <f>'Revenue Forecast'!K19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!K19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(K$3)-2026)</f>
         <v/>
       </c>
       <c r="L13" s="43">
-        <f>'Revenue Forecast'!L19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!L19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(L$3)-2026)</f>
         <v/>
       </c>
       <c r="M13" s="43">
-        <f>'Revenue Forecast'!M19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!M19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(M$3)-2026)</f>
         <v/>
       </c>
       <c r="N13" s="43">
-        <f>'Revenue Forecast'!N19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!N19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(N$3)-2026)</f>
         <v/>
       </c>
       <c r="O13" s="43">
-        <f>'Revenue Forecast'!O19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!O19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(O$3)-2026)</f>
         <v/>
       </c>
       <c r="P13" s="43">
-        <f>'Revenue Forecast'!P19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!P19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(P$3)-2026)</f>
         <v/>
       </c>
       <c r="Q13" s="43">
-        <f>'Revenue Forecast'!Q19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!Q19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(Q$3)-2026)</f>
         <v/>
       </c>
       <c r="R13" s="43">
-        <f>'Revenue Forecast'!R19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!R19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(R$3)-2026)</f>
         <v/>
       </c>
       <c r="S13" s="43">
-        <f>'Revenue Forecast'!S19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!S19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(S$3)-2026)</f>
         <v/>
       </c>
       <c r="T13" s="43">
-        <f>'Revenue Forecast'!T19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!T19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(T$3)-2026)</f>
         <v/>
       </c>
       <c r="U13" s="43">
-        <f>'Revenue Forecast'!U19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!U19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(U$3)-2026)</f>
         <v/>
       </c>
       <c r="V13" s="43">
-        <f>'Revenue Forecast'!V19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!V19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(V$3)-2026)</f>
         <v/>
       </c>
       <c r="W13" s="43">
-        <f>'Revenue Forecast'!W19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!W19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(W$3)-2026)</f>
         <v/>
       </c>
       <c r="X13" s="43">
-        <f>'Revenue Forecast'!X19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!X19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(X$3)-2026)</f>
         <v/>
       </c>
       <c r="Y13" s="43">
-        <f>'Revenue Forecast'!Y19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!Y19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(Y$3)-2026)</f>
         <v/>
       </c>
       <c r="Z13" s="43">
-        <f>'Revenue Forecast'!Z19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!Z19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(Z$3)-2026)</f>
         <v/>
       </c>
       <c r="AA13" s="43">
-        <f>'Revenue Forecast'!AA19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AA19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AA$3)-2026)</f>
         <v/>
       </c>
       <c r="AB13" s="43">
-        <f>'Revenue Forecast'!AB19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AB19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AB$3)-2026)</f>
         <v/>
       </c>
       <c r="AC13" s="43">
-        <f>'Revenue Forecast'!AC19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AC19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AC$3)-2026)</f>
         <v/>
       </c>
       <c r="AD13" s="43">
-        <f>'Revenue Forecast'!AD19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AD19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AD$3)-2026)</f>
         <v/>
       </c>
       <c r="AE13" s="43">
-        <f>'Revenue Forecast'!AE19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AE19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AE$3)-2026)</f>
         <v/>
       </c>
       <c r="AF13" s="43">
-        <f>'Revenue Forecast'!AF19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AF19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AF$3)-2026)</f>
         <v/>
       </c>
       <c r="AG13" s="43">
-        <f>'Revenue Forecast'!AG19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AG19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AG$3)-2026)</f>
         <v/>
       </c>
       <c r="AH13" s="43">
-        <f>'Revenue Forecast'!AH19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AH19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AH$3)-2026)</f>
         <v/>
       </c>
       <c r="AI13" s="43">
-        <f>'Revenue Forecast'!AI19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AI19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AI$3)-2026)</f>
         <v/>
       </c>
       <c r="AJ13" s="43">
-        <f>'Revenue Forecast'!AJ19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AJ19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AJ$3)-2026)</f>
         <v/>
       </c>
       <c r="AK13" s="43">
-        <f>'Revenue Forecast'!AK19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AK19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AK$3)-2026)</f>
         <v/>
       </c>
       <c r="AL13" s="43">
-        <f>'Revenue Forecast'!AL19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AL19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AL$3)-2026)</f>
         <v/>
       </c>
       <c r="AM13" s="43">
-        <f>'Revenue Forecast'!AM19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AM19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AM$3)-2026)</f>
         <v/>
       </c>
       <c r="AN13" s="43">
-        <f>'Revenue Forecast'!AN19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AN19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AN$3)-2026)</f>
         <v/>
       </c>
       <c r="AO13" s="43">
-        <f>'Revenue Forecast'!AO19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AO19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AO$3)-2026)</f>
         <v/>
       </c>
       <c r="AP13" s="43">
-        <f>'Revenue Forecast'!AP19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AP19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AP$3)-2026)</f>
         <v/>
       </c>
       <c r="AQ13" s="43">
-        <f>'Revenue Forecast'!AQ19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AQ19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AQ$3)-2026)</f>
         <v/>
       </c>
       <c r="AR13" s="43">
-        <f>'Revenue Forecast'!AR19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AR19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AR$3)-2026)</f>
         <v/>
       </c>
       <c r="AS13" s="43">
-        <f>'Revenue Forecast'!AS19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AS19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AS$3)-2026)</f>
         <v/>
       </c>
       <c r="AT13" s="43">
-        <f>'Revenue Forecast'!AT19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AT19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AT$3)-2026)</f>
         <v/>
       </c>
       <c r="AU13" s="43">
-        <f>'Revenue Forecast'!AU19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AU19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AU$3)-2026)</f>
         <v/>
       </c>
       <c r="AV13" s="43">
-        <f>'Revenue Forecast'!AV19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AV19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AV$3)-2026)</f>
         <v/>
       </c>
       <c r="AW13" s="43">
-        <f>'Revenue Forecast'!AW19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AW19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AW$3)-2026)</f>
         <v/>
       </c>
       <c r="AX13" s="43">
-        <f>'Revenue Forecast'!AX19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AX19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AX$3)-2026)</f>
         <v/>
       </c>
       <c r="AY13" s="43">
-        <f>'Revenue Forecast'!AY19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AY19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AY$3)-2026)</f>
         <v/>
       </c>
       <c r="AZ13" s="43">
-        <f>'Revenue Forecast'!AZ19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!AZ19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(AZ$3)-2026)</f>
         <v/>
       </c>
       <c r="BA13" s="43">
-        <f>'Revenue Forecast'!BA19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!BA19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(BA$3)-2026)</f>
         <v/>
       </c>
       <c r="BB13" s="43">
-        <f>'Revenue Forecast'!BB19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!BB19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(BB$3)-2026)</f>
         <v/>
       </c>
       <c r="BC13" s="43">
-        <f>'Revenue Forecast'!BC19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!BC19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(BC$3)-2026)</f>
         <v/>
       </c>
       <c r="BD13" s="43">
-        <f>'Revenue Forecast'!BD19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!BD19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(BD$3)-2026)</f>
         <v/>
       </c>
       <c r="BE13" s="43">
-        <f>'Revenue Forecast'!BE19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!BE19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(BE$3)-2026)</f>
         <v/>
       </c>
       <c r="BF13" s="43">
-        <f>'Revenue Forecast'!BF19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!BF19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(BF$3)-2026)</f>
         <v/>
       </c>
       <c r="BG13" s="43">
-        <f>'Revenue Forecast'!BG19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!BG19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(BG$3)-2026)</f>
         <v/>
       </c>
       <c r="BH13" s="43">
-        <f>'Revenue Forecast'!BH19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!BH19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(BH$3)-2026)</f>
         <v/>
       </c>
       <c r="BI13" s="43">
-        <f>'Revenue Forecast'!BI19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!BI19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(BI$3)-2026)</f>
         <v/>
       </c>
       <c r="BJ13" s="43">
-        <f>'Revenue Forecast'!BJ19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!BJ19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(BJ$3)-2026)</f>
         <v/>
       </c>
       <c r="BK13" s="43">
-        <f>'Revenue Forecast'!BK19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!BK19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(BK$3)-2026)</f>
         <v/>
       </c>
       <c r="BL13" s="43">
-        <f>'Revenue Forecast'!BL19*Assumptions!$F$130</f>
+        <f>'Revenue Forecast'!BL19*Assumptions!$F$130*(1+Assumptions!$F$135)^(YEAR(BL$3)-2026)</f>
         <v/>
       </c>
       <c r="BN13" s="44">
@@ -35915,243 +35920,243 @@
         </is>
       </c>
       <c r="E22" s="43">
-        <f>Personnel!E20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!E20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(E$3)-2026)</f>
         <v/>
       </c>
       <c r="F22" s="43">
-        <f>Personnel!F20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!F20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(F$3)-2026)</f>
         <v/>
       </c>
       <c r="G22" s="43">
-        <f>Personnel!G20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!G20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(G$3)-2026)</f>
         <v/>
       </c>
       <c r="H22" s="43">
-        <f>Personnel!H20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!H20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(H$3)-2026)</f>
         <v/>
       </c>
       <c r="I22" s="43">
-        <f>Personnel!I20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!I20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(I$3)-2026)</f>
         <v/>
       </c>
       <c r="J22" s="43">
-        <f>Personnel!J20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!J20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(J$3)-2026)</f>
         <v/>
       </c>
       <c r="K22" s="43">
-        <f>Personnel!K20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!K20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(K$3)-2026)</f>
         <v/>
       </c>
       <c r="L22" s="43">
-        <f>Personnel!L20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!L20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(L$3)-2026)</f>
         <v/>
       </c>
       <c r="M22" s="43">
-        <f>Personnel!M20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!M20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(M$3)-2026)</f>
         <v/>
       </c>
       <c r="N22" s="43">
-        <f>Personnel!N20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!N20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(N$3)-2026)</f>
         <v/>
       </c>
       <c r="O22" s="43">
-        <f>Personnel!O20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!O20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(O$3)-2026)</f>
         <v/>
       </c>
       <c r="P22" s="43">
-        <f>Personnel!P20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!P20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(P$3)-2026)</f>
         <v/>
       </c>
       <c r="Q22" s="43">
-        <f>Personnel!Q20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!Q20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(Q$3)-2026)</f>
         <v/>
       </c>
       <c r="R22" s="43">
-        <f>Personnel!R20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!R20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(R$3)-2026)</f>
         <v/>
       </c>
       <c r="S22" s="43">
-        <f>Personnel!S20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!S20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(S$3)-2026)</f>
         <v/>
       </c>
       <c r="T22" s="43">
-        <f>Personnel!T20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!T20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(T$3)-2026)</f>
         <v/>
       </c>
       <c r="U22" s="43">
-        <f>Personnel!U20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!U20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(U$3)-2026)</f>
         <v/>
       </c>
       <c r="V22" s="43">
-        <f>Personnel!V20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!V20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(V$3)-2026)</f>
         <v/>
       </c>
       <c r="W22" s="43">
-        <f>Personnel!W20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!W20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(W$3)-2026)</f>
         <v/>
       </c>
       <c r="X22" s="43">
-        <f>Personnel!X20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!X20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(X$3)-2026)</f>
         <v/>
       </c>
       <c r="Y22" s="43">
-        <f>Personnel!Y20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!Y20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(Y$3)-2026)</f>
         <v/>
       </c>
       <c r="Z22" s="43">
-        <f>Personnel!Z20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!Z20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(Z$3)-2026)</f>
         <v/>
       </c>
       <c r="AA22" s="43">
-        <f>Personnel!AA20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AA20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AA$3)-2026)</f>
         <v/>
       </c>
       <c r="AB22" s="43">
-        <f>Personnel!AB20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AB20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AB$3)-2026)</f>
         <v/>
       </c>
       <c r="AC22" s="43">
-        <f>Personnel!AC20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AC20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AC$3)-2026)</f>
         <v/>
       </c>
       <c r="AD22" s="43">
-        <f>Personnel!AD20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AD20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AD$3)-2026)</f>
         <v/>
       </c>
       <c r="AE22" s="43">
-        <f>Personnel!AE20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AE20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AE$3)-2026)</f>
         <v/>
       </c>
       <c r="AF22" s="43">
-        <f>Personnel!AF20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AF20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AF$3)-2026)</f>
         <v/>
       </c>
       <c r="AG22" s="43">
-        <f>Personnel!AG20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AG20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AG$3)-2026)</f>
         <v/>
       </c>
       <c r="AH22" s="43">
-        <f>Personnel!AH20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AH20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AH$3)-2026)</f>
         <v/>
       </c>
       <c r="AI22" s="43">
-        <f>Personnel!AI20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AI20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AI$3)-2026)</f>
         <v/>
       </c>
       <c r="AJ22" s="43">
-        <f>Personnel!AJ20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AJ20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AJ$3)-2026)</f>
         <v/>
       </c>
       <c r="AK22" s="43">
-        <f>Personnel!AK20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AK20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AK$3)-2026)</f>
         <v/>
       </c>
       <c r="AL22" s="43">
-        <f>Personnel!AL20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AL20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AL$3)-2026)</f>
         <v/>
       </c>
       <c r="AM22" s="43">
-        <f>Personnel!AM20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AM20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AM$3)-2026)</f>
         <v/>
       </c>
       <c r="AN22" s="43">
-        <f>Personnel!AN20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AN20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AN$3)-2026)</f>
         <v/>
       </c>
       <c r="AO22" s="43">
-        <f>Personnel!AO20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AO20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AO$3)-2026)</f>
         <v/>
       </c>
       <c r="AP22" s="43">
-        <f>Personnel!AP20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AP20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AP$3)-2026)</f>
         <v/>
       </c>
       <c r="AQ22" s="43">
-        <f>Personnel!AQ20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AQ20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AQ$3)-2026)</f>
         <v/>
       </c>
       <c r="AR22" s="43">
-        <f>Personnel!AR20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AR20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AR$3)-2026)</f>
         <v/>
       </c>
       <c r="AS22" s="43">
-        <f>Personnel!AS20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AS20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AS$3)-2026)</f>
         <v/>
       </c>
       <c r="AT22" s="43">
-        <f>Personnel!AT20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AT20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AT$3)-2026)</f>
         <v/>
       </c>
       <c r="AU22" s="43">
-        <f>Personnel!AU20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AU20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AU$3)-2026)</f>
         <v/>
       </c>
       <c r="AV22" s="43">
-        <f>Personnel!AV20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AV20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AV$3)-2026)</f>
         <v/>
       </c>
       <c r="AW22" s="43">
-        <f>Personnel!AW20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AW20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AW$3)-2026)</f>
         <v/>
       </c>
       <c r="AX22" s="43">
-        <f>Personnel!AX20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AX20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AX$3)-2026)</f>
         <v/>
       </c>
       <c r="AY22" s="43">
-        <f>Personnel!AY20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AY20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AY$3)-2026)</f>
         <v/>
       </c>
       <c r="AZ22" s="43">
-        <f>Personnel!AZ20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!AZ20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(AZ$3)-2026)</f>
         <v/>
       </c>
       <c r="BA22" s="43">
-        <f>Personnel!BA20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!BA20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(BA$3)-2026)</f>
         <v/>
       </c>
       <c r="BB22" s="43">
-        <f>Personnel!BB20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!BB20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(BB$3)-2026)</f>
         <v/>
       </c>
       <c r="BC22" s="43">
-        <f>Personnel!BC20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!BC20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(BC$3)-2026)</f>
         <v/>
       </c>
       <c r="BD22" s="43">
-        <f>Personnel!BD20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!BD20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(BD$3)-2026)</f>
         <v/>
       </c>
       <c r="BE22" s="43">
-        <f>Personnel!BE20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!BE20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(BE$3)-2026)</f>
         <v/>
       </c>
       <c r="BF22" s="43">
-        <f>Personnel!BF20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!BF20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(BF$3)-2026)</f>
         <v/>
       </c>
       <c r="BG22" s="43">
-        <f>Personnel!BG20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!BG20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(BG$3)-2026)</f>
         <v/>
       </c>
       <c r="BH22" s="43">
-        <f>Personnel!BH20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!BH20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(BH$3)-2026)</f>
         <v/>
       </c>
       <c r="BI22" s="43">
-        <f>Personnel!BI20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!BI20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(BI$3)-2026)</f>
         <v/>
       </c>
       <c r="BJ22" s="43">
-        <f>Personnel!BJ20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!BJ20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(BJ$3)-2026)</f>
         <v/>
       </c>
       <c r="BK22" s="43">
-        <f>Personnel!BK20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!BK20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(BK$3)-2026)</f>
         <v/>
       </c>
       <c r="BL22" s="43">
-        <f>Personnel!BL20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)</f>
+        <f>Personnel!BL20*(Assumptions!$F$126+Assumptions!$F$127+Assumptions!$F$128)*(1+Assumptions!$F$135)^(YEAR(BL$3)-2026)</f>
         <v/>
       </c>
       <c r="BN22" s="44">
@@ -36176,7 +36181,7 @@
       </c>
       <c r="BT22" s="20" t="inlineStr">
         <is>
-          <t>scales with the number of people on the payroll</t>
+          <t>scales with the number of people on the payroll, inflated like every other cost</t>
         </is>
       </c>
     </row>
@@ -36196,239 +36201,239 @@
         <v/>
       </c>
       <c r="F23" s="43">
-        <f>MAX(0,Personnel!F20-Personnel!E20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!F20-Personnel!E20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(F$3)-2026)</f>
         <v/>
       </c>
       <c r="G23" s="43">
-        <f>MAX(0,Personnel!G20-Personnel!F20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!G20-Personnel!F20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(G$3)-2026)</f>
         <v/>
       </c>
       <c r="H23" s="43">
-        <f>MAX(0,Personnel!H20-Personnel!G20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!H20-Personnel!G20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(H$3)-2026)</f>
         <v/>
       </c>
       <c r="I23" s="43">
-        <f>MAX(0,Personnel!I20-Personnel!H20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!I20-Personnel!H20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(I$3)-2026)</f>
         <v/>
       </c>
       <c r="J23" s="43">
-        <f>MAX(0,Personnel!J20-Personnel!I20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!J20-Personnel!I20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(J$3)-2026)</f>
         <v/>
       </c>
       <c r="K23" s="43">
-        <f>MAX(0,Personnel!K20-Personnel!J20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!K20-Personnel!J20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(K$3)-2026)</f>
         <v/>
       </c>
       <c r="L23" s="43">
-        <f>MAX(0,Personnel!L20-Personnel!K20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!L20-Personnel!K20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(L$3)-2026)</f>
         <v/>
       </c>
       <c r="M23" s="43">
-        <f>MAX(0,Personnel!M20-Personnel!L20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!M20-Personnel!L20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(M$3)-2026)</f>
         <v/>
       </c>
       <c r="N23" s="43">
-        <f>MAX(0,Personnel!N20-Personnel!M20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!N20-Personnel!M20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(N$3)-2026)</f>
         <v/>
       </c>
       <c r="O23" s="43">
-        <f>MAX(0,Personnel!O20-Personnel!N20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!O20-Personnel!N20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(O$3)-2026)</f>
         <v/>
       </c>
       <c r="P23" s="43">
-        <f>MAX(0,Personnel!P20-Personnel!O20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!P20-Personnel!O20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(P$3)-2026)</f>
         <v/>
       </c>
       <c r="Q23" s="43">
-        <f>MAX(0,Personnel!Q20-Personnel!P20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!Q20-Personnel!P20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(Q$3)-2026)</f>
         <v/>
       </c>
       <c r="R23" s="43">
-        <f>MAX(0,Personnel!R20-Personnel!Q20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!R20-Personnel!Q20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(R$3)-2026)</f>
         <v/>
       </c>
       <c r="S23" s="43">
-        <f>MAX(0,Personnel!S20-Personnel!R20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!S20-Personnel!R20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(S$3)-2026)</f>
         <v/>
       </c>
       <c r="T23" s="43">
-        <f>MAX(0,Personnel!T20-Personnel!S20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!T20-Personnel!S20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(T$3)-2026)</f>
         <v/>
       </c>
       <c r="U23" s="43">
-        <f>MAX(0,Personnel!U20-Personnel!T20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!U20-Personnel!T20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(U$3)-2026)</f>
         <v/>
       </c>
       <c r="V23" s="43">
-        <f>MAX(0,Personnel!V20-Personnel!U20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!V20-Personnel!U20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(V$3)-2026)</f>
         <v/>
       </c>
       <c r="W23" s="43">
-        <f>MAX(0,Personnel!W20-Personnel!V20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!W20-Personnel!V20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(W$3)-2026)</f>
         <v/>
       </c>
       <c r="X23" s="43">
-        <f>MAX(0,Personnel!X20-Personnel!W20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!X20-Personnel!W20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(X$3)-2026)</f>
         <v/>
       </c>
       <c r="Y23" s="43">
-        <f>MAX(0,Personnel!Y20-Personnel!X20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!Y20-Personnel!X20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(Y$3)-2026)</f>
         <v/>
       </c>
       <c r="Z23" s="43">
-        <f>MAX(0,Personnel!Z20-Personnel!Y20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!Z20-Personnel!Y20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(Z$3)-2026)</f>
         <v/>
       </c>
       <c r="AA23" s="43">
-        <f>MAX(0,Personnel!AA20-Personnel!Z20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AA20-Personnel!Z20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AA$3)-2026)</f>
         <v/>
       </c>
       <c r="AB23" s="43">
-        <f>MAX(0,Personnel!AB20-Personnel!AA20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AB20-Personnel!AA20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AB$3)-2026)</f>
         <v/>
       </c>
       <c r="AC23" s="43">
-        <f>MAX(0,Personnel!AC20-Personnel!AB20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AC20-Personnel!AB20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AC$3)-2026)</f>
         <v/>
       </c>
       <c r="AD23" s="43">
-        <f>MAX(0,Personnel!AD20-Personnel!AC20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AD20-Personnel!AC20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AD$3)-2026)</f>
         <v/>
       </c>
       <c r="AE23" s="43">
-        <f>MAX(0,Personnel!AE20-Personnel!AD20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AE20-Personnel!AD20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AE$3)-2026)</f>
         <v/>
       </c>
       <c r="AF23" s="43">
-        <f>MAX(0,Personnel!AF20-Personnel!AE20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AF20-Personnel!AE20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AF$3)-2026)</f>
         <v/>
       </c>
       <c r="AG23" s="43">
-        <f>MAX(0,Personnel!AG20-Personnel!AF20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AG20-Personnel!AF20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AG$3)-2026)</f>
         <v/>
       </c>
       <c r="AH23" s="43">
-        <f>MAX(0,Personnel!AH20-Personnel!AG20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AH20-Personnel!AG20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AH$3)-2026)</f>
         <v/>
       </c>
       <c r="AI23" s="43">
-        <f>MAX(0,Personnel!AI20-Personnel!AH20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AI20-Personnel!AH20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AI$3)-2026)</f>
         <v/>
       </c>
       <c r="AJ23" s="43">
-        <f>MAX(0,Personnel!AJ20-Personnel!AI20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AJ20-Personnel!AI20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AJ$3)-2026)</f>
         <v/>
       </c>
       <c r="AK23" s="43">
-        <f>MAX(0,Personnel!AK20-Personnel!AJ20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AK20-Personnel!AJ20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AK$3)-2026)</f>
         <v/>
       </c>
       <c r="AL23" s="43">
-        <f>MAX(0,Personnel!AL20-Personnel!AK20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AL20-Personnel!AK20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AL$3)-2026)</f>
         <v/>
       </c>
       <c r="AM23" s="43">
-        <f>MAX(0,Personnel!AM20-Personnel!AL20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AM20-Personnel!AL20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AM$3)-2026)</f>
         <v/>
       </c>
       <c r="AN23" s="43">
-        <f>MAX(0,Personnel!AN20-Personnel!AM20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AN20-Personnel!AM20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AN$3)-2026)</f>
         <v/>
       </c>
       <c r="AO23" s="43">
-        <f>MAX(0,Personnel!AO20-Personnel!AN20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AO20-Personnel!AN20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AO$3)-2026)</f>
         <v/>
       </c>
       <c r="AP23" s="43">
-        <f>MAX(0,Personnel!AP20-Personnel!AO20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AP20-Personnel!AO20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AP$3)-2026)</f>
         <v/>
       </c>
       <c r="AQ23" s="43">
-        <f>MAX(0,Personnel!AQ20-Personnel!AP20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AQ20-Personnel!AP20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AQ$3)-2026)</f>
         <v/>
       </c>
       <c r="AR23" s="43">
-        <f>MAX(0,Personnel!AR20-Personnel!AQ20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AR20-Personnel!AQ20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AR$3)-2026)</f>
         <v/>
       </c>
       <c r="AS23" s="43">
-        <f>MAX(0,Personnel!AS20-Personnel!AR20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AS20-Personnel!AR20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AS$3)-2026)</f>
         <v/>
       </c>
       <c r="AT23" s="43">
-        <f>MAX(0,Personnel!AT20-Personnel!AS20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AT20-Personnel!AS20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AT$3)-2026)</f>
         <v/>
       </c>
       <c r="AU23" s="43">
-        <f>MAX(0,Personnel!AU20-Personnel!AT20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AU20-Personnel!AT20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AU$3)-2026)</f>
         <v/>
       </c>
       <c r="AV23" s="43">
-        <f>MAX(0,Personnel!AV20-Personnel!AU20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AV20-Personnel!AU20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AV$3)-2026)</f>
         <v/>
       </c>
       <c r="AW23" s="43">
-        <f>MAX(0,Personnel!AW20-Personnel!AV20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AW20-Personnel!AV20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AW$3)-2026)</f>
         <v/>
       </c>
       <c r="AX23" s="43">
-        <f>MAX(0,Personnel!AX20-Personnel!AW20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AX20-Personnel!AW20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AX$3)-2026)</f>
         <v/>
       </c>
       <c r="AY23" s="43">
-        <f>MAX(0,Personnel!AY20-Personnel!AX20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AY20-Personnel!AX20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AY$3)-2026)</f>
         <v/>
       </c>
       <c r="AZ23" s="43">
-        <f>MAX(0,Personnel!AZ20-Personnel!AY20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!AZ20-Personnel!AY20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(AZ$3)-2026)</f>
         <v/>
       </c>
       <c r="BA23" s="43">
-        <f>MAX(0,Personnel!BA20-Personnel!AZ20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!BA20-Personnel!AZ20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(BA$3)-2026)</f>
         <v/>
       </c>
       <c r="BB23" s="43">
-        <f>MAX(0,Personnel!BB20-Personnel!BA20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!BB20-Personnel!BA20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(BB$3)-2026)</f>
         <v/>
       </c>
       <c r="BC23" s="43">
-        <f>MAX(0,Personnel!BC20-Personnel!BB20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!BC20-Personnel!BB20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(BC$3)-2026)</f>
         <v/>
       </c>
       <c r="BD23" s="43">
-        <f>MAX(0,Personnel!BD20-Personnel!BC20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!BD20-Personnel!BC20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(BD$3)-2026)</f>
         <v/>
       </c>
       <c r="BE23" s="43">
-        <f>MAX(0,Personnel!BE20-Personnel!BD20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!BE20-Personnel!BD20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(BE$3)-2026)</f>
         <v/>
       </c>
       <c r="BF23" s="43">
-        <f>MAX(0,Personnel!BF20-Personnel!BE20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!BF20-Personnel!BE20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(BF$3)-2026)</f>
         <v/>
       </c>
       <c r="BG23" s="43">
-        <f>MAX(0,Personnel!BG20-Personnel!BF20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!BG20-Personnel!BF20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(BG$3)-2026)</f>
         <v/>
       </c>
       <c r="BH23" s="43">
-        <f>MAX(0,Personnel!BH20-Personnel!BG20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!BH20-Personnel!BG20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(BH$3)-2026)</f>
         <v/>
       </c>
       <c r="BI23" s="43">
-        <f>MAX(0,Personnel!BI20-Personnel!BH20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!BI20-Personnel!BH20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(BI$3)-2026)</f>
         <v/>
       </c>
       <c r="BJ23" s="43">
-        <f>MAX(0,Personnel!BJ20-Personnel!BI20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!BJ20-Personnel!BI20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(BJ$3)-2026)</f>
         <v/>
       </c>
       <c r="BK23" s="43">
-        <f>MAX(0,Personnel!BK20-Personnel!BJ20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!BK20-Personnel!BJ20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(BK$3)-2026)</f>
         <v/>
       </c>
       <c r="BL23" s="43">
-        <f>MAX(0,Personnel!BL20-Personnel!BK20)*Assumptions!$F$129</f>
+        <f>MAX(0,Personnel!BL20-Personnel!BK20)*Assumptions!$F$129*(1+Assumptions!$F$135)^(YEAR(BL$3)-2026)</f>
         <v/>
       </c>
       <c r="BN23" s="44">
@@ -38964,23 +38969,23 @@
         <v/>
       </c>
       <c r="BN35" s="49">
-        <f>IFERROR(AVERAGE(E35:P35),0)</f>
+        <f>IFERROR(BN33/'Revenue Forecast'!BN50,0)</f>
         <v/>
       </c>
       <c r="BO35" s="49">
-        <f>IFERROR(AVERAGE(Q35:AB35),0)</f>
+        <f>IFERROR(BO33/'Revenue Forecast'!BO50,0)</f>
         <v/>
       </c>
       <c r="BP35" s="49">
-        <f>IFERROR(AVERAGE(AC35:AN35),0)</f>
+        <f>IFERROR(BP33/'Revenue Forecast'!BP50,0)</f>
         <v/>
       </c>
       <c r="BQ35" s="49">
-        <f>IFERROR(AVERAGE(AO35:AZ35),0)</f>
+        <f>IFERROR(BQ33/'Revenue Forecast'!BQ50,0)</f>
         <v/>
       </c>
       <c r="BR35" s="49">
-        <f>IFERROR(AVERAGE(BA35:BL35),0)</f>
+        <f>IFERROR(BR33/'Revenue Forecast'!BR50,0)</f>
         <v/>
       </c>
     </row>
@@ -39101,156 +39106,56 @@
       <c r="N38" s="23" t="n">
         <v>61620</v>
       </c>
-      <c r="O38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="S38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="T38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="U38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="V38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="W38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="X38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL38" s="23" t="n">
-        <v>0</v>
-      </c>
+      <c r="O38" s="43" t="n"/>
+      <c r="P38" s="43" t="n"/>
+      <c r="Q38" s="43" t="n"/>
+      <c r="R38" s="43" t="n"/>
+      <c r="S38" s="43" t="n"/>
+      <c r="T38" s="43" t="n"/>
+      <c r="U38" s="43" t="n"/>
+      <c r="V38" s="43" t="n"/>
+      <c r="W38" s="43" t="n"/>
+      <c r="X38" s="43" t="n"/>
+      <c r="Y38" s="43" t="n"/>
+      <c r="Z38" s="43" t="n"/>
+      <c r="AA38" s="43" t="n"/>
+      <c r="AB38" s="43" t="n"/>
+      <c r="AC38" s="43" t="n"/>
+      <c r="AD38" s="43" t="n"/>
+      <c r="AE38" s="43" t="n"/>
+      <c r="AF38" s="43" t="n"/>
+      <c r="AG38" s="43" t="n"/>
+      <c r="AH38" s="43" t="n"/>
+      <c r="AI38" s="43" t="n"/>
+      <c r="AJ38" s="43" t="n"/>
+      <c r="AK38" s="43" t="n"/>
+      <c r="AL38" s="43" t="n"/>
+      <c r="AM38" s="43" t="n"/>
+      <c r="AN38" s="43" t="n"/>
+      <c r="AO38" s="43" t="n"/>
+      <c r="AP38" s="43" t="n"/>
+      <c r="AQ38" s="43" t="n"/>
+      <c r="AR38" s="43" t="n"/>
+      <c r="AS38" s="43" t="n"/>
+      <c r="AT38" s="43" t="n"/>
+      <c r="AU38" s="43" t="n"/>
+      <c r="AV38" s="43" t="n"/>
+      <c r="AW38" s="43" t="n"/>
+      <c r="AX38" s="43" t="n"/>
+      <c r="AY38" s="43" t="n"/>
+      <c r="AZ38" s="43" t="n"/>
+      <c r="BA38" s="43" t="n"/>
+      <c r="BB38" s="43" t="n"/>
+      <c r="BC38" s="43" t="n"/>
+      <c r="BD38" s="43" t="n"/>
+      <c r="BE38" s="43" t="n"/>
+      <c r="BF38" s="43" t="n"/>
+      <c r="BG38" s="43" t="n"/>
+      <c r="BH38" s="43" t="n"/>
+      <c r="BI38" s="43" t="n"/>
+      <c r="BJ38" s="43" t="n"/>
+      <c r="BK38" s="43" t="n"/>
+      <c r="BL38" s="43" t="n"/>
       <c r="BN38" s="44">
         <f>SUM(E38:P38)</f>
         <v/>
@@ -39318,156 +39223,56 @@
       <c r="N39" s="23" t="n">
         <v>19800</v>
       </c>
-      <c r="O39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="S39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="T39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="U39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="V39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="W39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="X39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL39" s="23" t="n">
-        <v>0</v>
-      </c>
+      <c r="O39" s="43" t="n"/>
+      <c r="P39" s="43" t="n"/>
+      <c r="Q39" s="43" t="n"/>
+      <c r="R39" s="43" t="n"/>
+      <c r="S39" s="43" t="n"/>
+      <c r="T39" s="43" t="n"/>
+      <c r="U39" s="43" t="n"/>
+      <c r="V39" s="43" t="n"/>
+      <c r="W39" s="43" t="n"/>
+      <c r="X39" s="43" t="n"/>
+      <c r="Y39" s="43" t="n"/>
+      <c r="Z39" s="43" t="n"/>
+      <c r="AA39" s="43" t="n"/>
+      <c r="AB39" s="43" t="n"/>
+      <c r="AC39" s="43" t="n"/>
+      <c r="AD39" s="43" t="n"/>
+      <c r="AE39" s="43" t="n"/>
+      <c r="AF39" s="43" t="n"/>
+      <c r="AG39" s="43" t="n"/>
+      <c r="AH39" s="43" t="n"/>
+      <c r="AI39" s="43" t="n"/>
+      <c r="AJ39" s="43" t="n"/>
+      <c r="AK39" s="43" t="n"/>
+      <c r="AL39" s="43" t="n"/>
+      <c r="AM39" s="43" t="n"/>
+      <c r="AN39" s="43" t="n"/>
+      <c r="AO39" s="43" t="n"/>
+      <c r="AP39" s="43" t="n"/>
+      <c r="AQ39" s="43" t="n"/>
+      <c r="AR39" s="43" t="n"/>
+      <c r="AS39" s="43" t="n"/>
+      <c r="AT39" s="43" t="n"/>
+      <c r="AU39" s="43" t="n"/>
+      <c r="AV39" s="43" t="n"/>
+      <c r="AW39" s="43" t="n"/>
+      <c r="AX39" s="43" t="n"/>
+      <c r="AY39" s="43" t="n"/>
+      <c r="AZ39" s="43" t="n"/>
+      <c r="BA39" s="43" t="n"/>
+      <c r="BB39" s="43" t="n"/>
+      <c r="BC39" s="43" t="n"/>
+      <c r="BD39" s="43" t="n"/>
+      <c r="BE39" s="43" t="n"/>
+      <c r="BF39" s="43" t="n"/>
+      <c r="BG39" s="43" t="n"/>
+      <c r="BH39" s="43" t="n"/>
+      <c r="BI39" s="43" t="n"/>
+      <c r="BJ39" s="43" t="n"/>
+      <c r="BK39" s="43" t="n"/>
+      <c r="BL39" s="43" t="n"/>
       <c r="BN39" s="44">
         <f>SUM(E39:P39)</f>
         <v/>
@@ -39530,156 +39335,56 @@
       <c r="N40" s="23" t="n">
         <v>21420</v>
       </c>
-      <c r="O40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="S40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="T40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="U40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="V40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="W40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="X40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL40" s="23" t="n">
-        <v>0</v>
-      </c>
+      <c r="O40" s="43" t="n"/>
+      <c r="P40" s="43" t="n"/>
+      <c r="Q40" s="43" t="n"/>
+      <c r="R40" s="43" t="n"/>
+      <c r="S40" s="43" t="n"/>
+      <c r="T40" s="43" t="n"/>
+      <c r="U40" s="43" t="n"/>
+      <c r="V40" s="43" t="n"/>
+      <c r="W40" s="43" t="n"/>
+      <c r="X40" s="43" t="n"/>
+      <c r="Y40" s="43" t="n"/>
+      <c r="Z40" s="43" t="n"/>
+      <c r="AA40" s="43" t="n"/>
+      <c r="AB40" s="43" t="n"/>
+      <c r="AC40" s="43" t="n"/>
+      <c r="AD40" s="43" t="n"/>
+      <c r="AE40" s="43" t="n"/>
+      <c r="AF40" s="43" t="n"/>
+      <c r="AG40" s="43" t="n"/>
+      <c r="AH40" s="43" t="n"/>
+      <c r="AI40" s="43" t="n"/>
+      <c r="AJ40" s="43" t="n"/>
+      <c r="AK40" s="43" t="n"/>
+      <c r="AL40" s="43" t="n"/>
+      <c r="AM40" s="43" t="n"/>
+      <c r="AN40" s="43" t="n"/>
+      <c r="AO40" s="43" t="n"/>
+      <c r="AP40" s="43" t="n"/>
+      <c r="AQ40" s="43" t="n"/>
+      <c r="AR40" s="43" t="n"/>
+      <c r="AS40" s="43" t="n"/>
+      <c r="AT40" s="43" t="n"/>
+      <c r="AU40" s="43" t="n"/>
+      <c r="AV40" s="43" t="n"/>
+      <c r="AW40" s="43" t="n"/>
+      <c r="AX40" s="43" t="n"/>
+      <c r="AY40" s="43" t="n"/>
+      <c r="AZ40" s="43" t="n"/>
+      <c r="BA40" s="43" t="n"/>
+      <c r="BB40" s="43" t="n"/>
+      <c r="BC40" s="43" t="n"/>
+      <c r="BD40" s="43" t="n"/>
+      <c r="BE40" s="43" t="n"/>
+      <c r="BF40" s="43" t="n"/>
+      <c r="BG40" s="43" t="n"/>
+      <c r="BH40" s="43" t="n"/>
+      <c r="BI40" s="43" t="n"/>
+      <c r="BJ40" s="43" t="n"/>
+      <c r="BK40" s="43" t="n"/>
+      <c r="BL40" s="43" t="n"/>
       <c r="BN40" s="44">
         <f>SUM(E40:P40)</f>
         <v/>
@@ -39742,156 +39447,56 @@
       <c r="N41" s="23" t="n">
         <v>125000</v>
       </c>
-      <c r="O41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="S41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="T41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="U41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="V41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="W41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="X41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL41" s="23" t="n">
-        <v>0</v>
-      </c>
+      <c r="O41" s="43" t="n"/>
+      <c r="P41" s="43" t="n"/>
+      <c r="Q41" s="43" t="n"/>
+      <c r="R41" s="43" t="n"/>
+      <c r="S41" s="43" t="n"/>
+      <c r="T41" s="43" t="n"/>
+      <c r="U41" s="43" t="n"/>
+      <c r="V41" s="43" t="n"/>
+      <c r="W41" s="43" t="n"/>
+      <c r="X41" s="43" t="n"/>
+      <c r="Y41" s="43" t="n"/>
+      <c r="Z41" s="43" t="n"/>
+      <c r="AA41" s="43" t="n"/>
+      <c r="AB41" s="43" t="n"/>
+      <c r="AC41" s="43" t="n"/>
+      <c r="AD41" s="43" t="n"/>
+      <c r="AE41" s="43" t="n"/>
+      <c r="AF41" s="43" t="n"/>
+      <c r="AG41" s="43" t="n"/>
+      <c r="AH41" s="43" t="n"/>
+      <c r="AI41" s="43" t="n"/>
+      <c r="AJ41" s="43" t="n"/>
+      <c r="AK41" s="43" t="n"/>
+      <c r="AL41" s="43" t="n"/>
+      <c r="AM41" s="43" t="n"/>
+      <c r="AN41" s="43" t="n"/>
+      <c r="AO41" s="43" t="n"/>
+      <c r="AP41" s="43" t="n"/>
+      <c r="AQ41" s="43" t="n"/>
+      <c r="AR41" s="43" t="n"/>
+      <c r="AS41" s="43" t="n"/>
+      <c r="AT41" s="43" t="n"/>
+      <c r="AU41" s="43" t="n"/>
+      <c r="AV41" s="43" t="n"/>
+      <c r="AW41" s="43" t="n"/>
+      <c r="AX41" s="43" t="n"/>
+      <c r="AY41" s="43" t="n"/>
+      <c r="AZ41" s="43" t="n"/>
+      <c r="BA41" s="43" t="n"/>
+      <c r="BB41" s="43" t="n"/>
+      <c r="BC41" s="43" t="n"/>
+      <c r="BD41" s="43" t="n"/>
+      <c r="BE41" s="43" t="n"/>
+      <c r="BF41" s="43" t="n"/>
+      <c r="BG41" s="43" t="n"/>
+      <c r="BH41" s="43" t="n"/>
+      <c r="BI41" s="43" t="n"/>
+      <c r="BJ41" s="43" t="n"/>
+      <c r="BK41" s="43" t="n"/>
+      <c r="BL41" s="43" t="n"/>
       <c r="BN41" s="44">
         <f>SUM(E41:P41)</f>
         <v/>
@@ -39954,156 +39559,56 @@
       <c r="N42" s="23" t="n">
         <v>24000</v>
       </c>
-      <c r="O42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="S42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="T42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="U42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="V42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="W42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="X42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL42" s="23" t="n">
-        <v>0</v>
-      </c>
+      <c r="O42" s="43" t="n"/>
+      <c r="P42" s="43" t="n"/>
+      <c r="Q42" s="43" t="n"/>
+      <c r="R42" s="43" t="n"/>
+      <c r="S42" s="43" t="n"/>
+      <c r="T42" s="43" t="n"/>
+      <c r="U42" s="43" t="n"/>
+      <c r="V42" s="43" t="n"/>
+      <c r="W42" s="43" t="n"/>
+      <c r="X42" s="43" t="n"/>
+      <c r="Y42" s="43" t="n"/>
+      <c r="Z42" s="43" t="n"/>
+      <c r="AA42" s="43" t="n"/>
+      <c r="AB42" s="43" t="n"/>
+      <c r="AC42" s="43" t="n"/>
+      <c r="AD42" s="43" t="n"/>
+      <c r="AE42" s="43" t="n"/>
+      <c r="AF42" s="43" t="n"/>
+      <c r="AG42" s="43" t="n"/>
+      <c r="AH42" s="43" t="n"/>
+      <c r="AI42" s="43" t="n"/>
+      <c r="AJ42" s="43" t="n"/>
+      <c r="AK42" s="43" t="n"/>
+      <c r="AL42" s="43" t="n"/>
+      <c r="AM42" s="43" t="n"/>
+      <c r="AN42" s="43" t="n"/>
+      <c r="AO42" s="43" t="n"/>
+      <c r="AP42" s="43" t="n"/>
+      <c r="AQ42" s="43" t="n"/>
+      <c r="AR42" s="43" t="n"/>
+      <c r="AS42" s="43" t="n"/>
+      <c r="AT42" s="43" t="n"/>
+      <c r="AU42" s="43" t="n"/>
+      <c r="AV42" s="43" t="n"/>
+      <c r="AW42" s="43" t="n"/>
+      <c r="AX42" s="43" t="n"/>
+      <c r="AY42" s="43" t="n"/>
+      <c r="AZ42" s="43" t="n"/>
+      <c r="BA42" s="43" t="n"/>
+      <c r="BB42" s="43" t="n"/>
+      <c r="BC42" s="43" t="n"/>
+      <c r="BD42" s="43" t="n"/>
+      <c r="BE42" s="43" t="n"/>
+      <c r="BF42" s="43" t="n"/>
+      <c r="BG42" s="43" t="n"/>
+      <c r="BH42" s="43" t="n"/>
+      <c r="BI42" s="43" t="n"/>
+      <c r="BJ42" s="43" t="n"/>
+      <c r="BK42" s="43" t="n"/>
+      <c r="BL42" s="43" t="n"/>
       <c r="BN42" s="44">
         <f>SUM(E42:P42)</f>
         <v/>
@@ -40166,156 +39671,56 @@
       <c r="N43" s="23" t="n">
         <v>20000</v>
       </c>
-      <c r="O43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="S43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="T43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="U43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="V43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="W43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="X43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL43" s="23" t="n">
-        <v>0</v>
-      </c>
+      <c r="O43" s="43" t="n"/>
+      <c r="P43" s="43" t="n"/>
+      <c r="Q43" s="43" t="n"/>
+      <c r="R43" s="43" t="n"/>
+      <c r="S43" s="43" t="n"/>
+      <c r="T43" s="43" t="n"/>
+      <c r="U43" s="43" t="n"/>
+      <c r="V43" s="43" t="n"/>
+      <c r="W43" s="43" t="n"/>
+      <c r="X43" s="43" t="n"/>
+      <c r="Y43" s="43" t="n"/>
+      <c r="Z43" s="43" t="n"/>
+      <c r="AA43" s="43" t="n"/>
+      <c r="AB43" s="43" t="n"/>
+      <c r="AC43" s="43" t="n"/>
+      <c r="AD43" s="43" t="n"/>
+      <c r="AE43" s="43" t="n"/>
+      <c r="AF43" s="43" t="n"/>
+      <c r="AG43" s="43" t="n"/>
+      <c r="AH43" s="43" t="n"/>
+      <c r="AI43" s="43" t="n"/>
+      <c r="AJ43" s="43" t="n"/>
+      <c r="AK43" s="43" t="n"/>
+      <c r="AL43" s="43" t="n"/>
+      <c r="AM43" s="43" t="n"/>
+      <c r="AN43" s="43" t="n"/>
+      <c r="AO43" s="43" t="n"/>
+      <c r="AP43" s="43" t="n"/>
+      <c r="AQ43" s="43" t="n"/>
+      <c r="AR43" s="43" t="n"/>
+      <c r="AS43" s="43" t="n"/>
+      <c r="AT43" s="43" t="n"/>
+      <c r="AU43" s="43" t="n"/>
+      <c r="AV43" s="43" t="n"/>
+      <c r="AW43" s="43" t="n"/>
+      <c r="AX43" s="43" t="n"/>
+      <c r="AY43" s="43" t="n"/>
+      <c r="AZ43" s="43" t="n"/>
+      <c r="BA43" s="43" t="n"/>
+      <c r="BB43" s="43" t="n"/>
+      <c r="BC43" s="43" t="n"/>
+      <c r="BD43" s="43" t="n"/>
+      <c r="BE43" s="43" t="n"/>
+      <c r="BF43" s="43" t="n"/>
+      <c r="BG43" s="43" t="n"/>
+      <c r="BH43" s="43" t="n"/>
+      <c r="BI43" s="43" t="n"/>
+      <c r="BJ43" s="43" t="n"/>
+      <c r="BK43" s="43" t="n"/>
+      <c r="BL43" s="43" t="n"/>
       <c r="BN43" s="44">
         <f>SUM(E43:P43)</f>
         <v/>
@@ -46267,24 +45672,29 @@
         <v/>
       </c>
       <c r="BN31" s="66">
-        <f>IFERROR(AVERAGE(E31:P31),0)</f>
+        <f>IFERROR(BN29/12/BN20,0)</f>
         <v/>
       </c>
       <c r="BO31" s="66">
-        <f>IFERROR(AVERAGE(Q31:AB31),0)</f>
+        <f>IFERROR(BO29/12/BO20,0)</f>
         <v/>
       </c>
       <c r="BP31" s="66">
-        <f>IFERROR(AVERAGE(AC31:AN31),0)</f>
+        <f>IFERROR(BP29/12/BP20,0)</f>
         <v/>
       </c>
       <c r="BQ31" s="66">
-        <f>IFERROR(AVERAGE(AO31:AZ31),0)</f>
+        <f>IFERROR(BQ29/12/BQ20,0)</f>
         <v/>
       </c>
       <c r="BR31" s="66">
-        <f>IFERROR(AVERAGE(BA31:BL31),0)</f>
-        <v/>
+        <f>IFERROR(BR29/12/BR20,0)</f>
+        <v/>
+      </c>
+      <c r="BT31" s="20" t="inlineStr">
+        <is>
+          <t>annual column: the year's people cost over twelve, per head at December</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -46786,23 +46196,23 @@
         </is>
       </c>
       <c r="D26" s="43">
-        <f>IFERROR(D14/D25,0)</f>
+        <f>IFERROR(D14/D24,0)</f>
         <v/>
       </c>
       <c r="E26" s="43">
-        <f>IFERROR(E14/E25,0)</f>
+        <f>IFERROR(E14/E24,0)</f>
         <v/>
       </c>
       <c r="F26" s="43">
-        <f>IFERROR(F14/F25,0)</f>
+        <f>IFERROR(F14/F24,0)</f>
         <v/>
       </c>
       <c r="G26" s="43">
-        <f>IFERROR(G14/G25,0)</f>
+        <f>IFERROR(G14/G24,0)</f>
         <v/>
       </c>
       <c r="H26" s="43">
-        <f>IFERROR(H14/H25,0)</f>
+        <f>IFERROR(H14/H24,0)</f>
         <v/>
       </c>
       <c r="J26" s="20" t="inlineStr">
@@ -46977,7 +46387,7 @@
         </is>
       </c>
       <c r="D37" s="43">
-        <f>MIN('Financial Statements'!$N$40:$BL$40)</f>
+        <f>MIN(INDEX('Financial Statements'!$E$40:$BL$40,MATCH(Assumptions!$F$140,'Financial Statements'!$E$3:$BL$3,0)):INDEX('Financial Statements'!$E$40:$BL$40,60))</f>
         <v/>
       </c>
       <c r="J37" s="20" t="inlineStr">
@@ -46993,7 +46403,7 @@
         </is>
       </c>
       <c r="D38" s="71">
-        <f>INDEX('Financial Statements'!$E$3:$BL$3,MATCH(D37,'Financial Statements'!$N$40:$BL$40,0)+9)</f>
+        <f>INDEX('Financial Statements'!$E$3:$BL$3,MATCH(D37,INDEX('Financial Statements'!$E$40:$BL$40,MATCH(Assumptions!$F$140,'Financial Statements'!$E$3:$BL$3,0)):INDEX('Financial Statements'!$E$40:$BL$40,60),0)+MATCH(Assumptions!$F$140,'Financial Statements'!$E$3:$BL$3,0)-1)</f>
         <v/>
       </c>
     </row>
@@ -47122,7 +46532,7 @@
         </is>
       </c>
       <c r="D50" s="43">
-        <f>'Financial Statements'!N40</f>
+        <f>INDEX('Financial Statements'!$E$40:$BL$40,MATCH(Assumptions!$F$140,'Financial Statements'!$E$3:$BL$3,0))</f>
         <v/>
       </c>
     </row>
@@ -47144,7 +46554,7 @@
         </is>
       </c>
       <c r="D52" s="72">
-        <f>IFERROR(D51/SUM('Financial Statements'!N35:BL35),0)</f>
+        <f>IFERROR(D51/SUM(INDEX('Financial Statements'!$E$35:$BL$35,MATCH(Assumptions!$F$140,'Financial Statements'!$E$3:$BL$3,0)):INDEX('Financial Statements'!$E$35:$BL$35,60)),0)</f>
         <v/>
       </c>
       <c r="J52" s="20" t="inlineStr">
@@ -47160,12 +46570,12 @@
         </is>
       </c>
       <c r="D53" s="60">
-        <f>IFERROR(D37/(-'Financial Statements'!BP14/12),0)</f>
+        <f>IFERROR(D37/(-HLOOKUP(YEAR(D38),'Financial Statements'!$BN$3:$BR$14,12,FALSE)/12),0)</f>
         <v/>
       </c>
       <c r="J53" s="20" t="inlineStr">
         <is>
-          <t>a plan of this size wants three months or more here</t>
+          <t>cash at the low point over that year's average monthly operating cost. Three months or more is comfortable</t>
         </is>
       </c>
     </row>

</xml_diff>